<commit_message>
FIx A6 decline data
</commit_message>
<xml_diff>
--- a/data/S001.xlsx
+++ b/data/S001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://odsi2005-my.sharepoint.com/personal/ibrahim_eltaleb_odsi-energy_com/Documents/ODSI_Desktop/Python/Stramlit/Dash_ODSI/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{6132AEC3-1CAB-4FBA-A026-50CE20EF1FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15C0DBDB-D79B-447D-80FF-A4CA545AAB37}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{6132AEC3-1CAB-4FBA-A026-50CE20EF1FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86AA71A3-6283-4AD6-9803-63D9253B0DBE}"/>
   <bookViews>
-    <workbookView xWindow="2616" yWindow="2616" windowWidth="23040" windowHeight="13608" xr2:uid="{92B28833-6805-4A4F-8867-695E222A4EA9}"/>
+    <workbookView xWindow="2616" yWindow="2616" windowWidth="23040" windowHeight="13608" activeTab="2" xr2:uid="{92B28833-6805-4A4F-8867-695E222A4EA9}"/>
   </bookViews>
   <sheets>
     <sheet name="EW A5 May 29-July 2026 1-min ex" sheetId="1" r:id="rId1"/>
@@ -448,7 +448,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="99">
   <si>
     <t>DateTime</t>
   </si>
@@ -705,9 +705,6 @@
     <t>S2</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>S3</t>
   </si>
   <si>
@@ -754,12 +751,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="mm/dd/yy;@"/>
     <numFmt numFmtId="167" formatCode="0.00000"/>
-    <numFmt numFmtId="168" formatCode="0.000000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -867,7 +863,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -914,7 +910,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -37282,7 +37277,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64D45957-36EC-4E57-B84E-45135FEB24AC}">
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -37406,947 +37401,1955 @@
       <c r="A5" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="2">
-        <v>46063.17423611111</v>
-      </c>
-      <c r="D5">
-        <v>21.84</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="F5">
-        <v>1340</v>
+      <c r="C5" s="20">
+        <v>44718</v>
+      </c>
+      <c r="D5" s="16">
+        <v>153.15</v>
+      </c>
+      <c r="E5" s="18">
+        <v>2.4510000000000001E-2</v>
+      </c>
+      <c r="F5" s="21">
+        <v>6450</v>
       </c>
       <c r="G5">
-        <v>11007</v>
+        <v>14640</v>
       </c>
       <c r="H5" s="19">
-        <v>5.3832101591728545E-6</v>
+        <v>6.5528873748480144E-6</v>
       </c>
       <c r="I5" s="19">
-        <v>1.9668247111420999E-5</v>
-      </c>
-      <c r="J5">
-        <v>8.6440000000000006E-3</v>
-      </c>
-      <c r="K5" s="18">
-        <v>1.5</v>
-      </c>
-      <c r="L5" s="18">
-        <f t="shared" ref="L5:L16" si="0">K5*0.325</f>
-        <v>0.48750000000000004</v>
+        <v>2.048702116239361E-5</v>
+      </c>
+      <c r="J5" s="16">
+        <v>3.8635999999999997E-2</v>
+      </c>
+      <c r="K5" s="16">
+        <v>2.0301248201269537</v>
+      </c>
+      <c r="L5" s="16">
+        <v>0.63594322154222771</v>
       </c>
       <c r="M5" s="16">
-        <f>K5*1.15</f>
-        <v>1.7249999999999999</v>
+        <v>2.0943556985273259</v>
       </c>
       <c r="N5" s="16">
-        <f t="shared" ref="N5:N16" si="1">M5*0.28</f>
-        <v>0.48299999999999998</v>
+        <v>0.65520798824681681</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" s="2">
-        <v>46080.991076388891</v>
-      </c>
-      <c r="D6">
-        <v>25.57</v>
-      </c>
-      <c r="E6" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="F6">
-        <v>1620</v>
+      <c r="C6" s="20">
+        <v>44743</v>
+      </c>
+      <c r="D6" s="16">
+        <v>48.3</v>
+      </c>
+      <c r="E6" s="18">
+        <v>1.2447E-2</v>
+      </c>
+      <c r="F6" s="21">
+        <v>5240</v>
       </c>
       <c r="G6">
-        <v>10983</v>
+        <v>13140</v>
       </c>
       <c r="H6" s="19">
-        <v>5.3928439229556913E-6</v>
+        <v>7.4641259754480077E-6</v>
       </c>
       <c r="I6" s="19">
-        <v>1.9674990746068985E-5</v>
-      </c>
-      <c r="J6">
-        <v>1.9238000000000002E-2</v>
-      </c>
-      <c r="K6" s="18">
-        <v>1.75</v>
-      </c>
-      <c r="L6" s="18">
-        <f t="shared" si="0"/>
-        <v>0.56874999999999998</v>
+        <v>2.1124888182813605E-5</v>
+      </c>
+      <c r="J6" s="16">
+        <v>0.20100000000000001</v>
+      </c>
+      <c r="K6" s="16">
+        <v>4.0041275544137367</v>
+      </c>
+      <c r="L6" s="16">
+        <v>1.2566760665220535</v>
       </c>
       <c r="M6" s="16">
-        <f t="shared" ref="M6:M17" si="2">K6*1.15</f>
-        <v>2.0124999999999997</v>
+        <v>5.3365828204904329</v>
       </c>
       <c r="N6" s="16">
-        <f t="shared" si="1"/>
-        <v>0.5635</v>
+        <v>1.6265403726708076</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" t="s">
         <v>87</v>
       </c>
-      <c r="B7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C7" s="2">
-        <v>46115.518842592595</v>
-      </c>
-      <c r="D7">
-        <v>4.6289999999999996</v>
-      </c>
-      <c r="E7" s="20">
-        <v>1.7957999999999998E-2</v>
-      </c>
-      <c r="F7">
-        <v>990</v>
+      <c r="C7" s="20">
+        <v>44761</v>
+      </c>
+      <c r="D7" s="16">
+        <v>31.57</v>
+      </c>
+      <c r="E7" s="18">
+        <v>1.0845E-2</v>
+      </c>
+      <c r="F7" s="21">
+        <v>4880</v>
       </c>
       <c r="G7">
-        <v>10868</v>
+        <v>12473</v>
       </c>
       <c r="H7" s="19">
-        <v>5.4396973008515152E-6</v>
+        <v>7.9061837905076426E-6</v>
       </c>
       <c r="I7" s="19">
-        <v>1.970778811059606E-5</v>
-      </c>
-      <c r="J7">
-        <v>5.5649999999999998E-2</v>
-      </c>
-      <c r="K7" s="18">
-        <v>2.8812074927656726</v>
-      </c>
-      <c r="L7" s="18">
-        <f t="shared" si="0"/>
-        <v>0.93639243514884363</v>
+        <v>2.1434328653355349E-5</v>
+      </c>
+      <c r="J7" s="16">
+        <v>0.29899999999999999</v>
+      </c>
+      <c r="K7" s="16">
+        <v>4.6009024507279497</v>
+      </c>
+      <c r="L7" s="16">
+        <v>1.4491152604887043</v>
       </c>
       <c r="M7" s="16">
-        <f t="shared" si="2"/>
-        <v>3.3133886166805233</v>
+        <v>7.5106618479995468</v>
       </c>
       <c r="N7" s="16">
-        <f t="shared" si="1"/>
-        <v>0.92774881267054665</v>
+        <v>2.2270405448210324</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" t="s">
         <v>89</v>
       </c>
-      <c r="B8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" s="2">
-        <v>46133.561631944445</v>
-      </c>
-      <c r="D8">
-        <v>5.7060000000000004</v>
+      <c r="C8" s="20">
+        <v>44778</v>
+      </c>
+      <c r="D8" s="16">
+        <v>23.65</v>
       </c>
       <c r="E8" s="18">
-        <v>3.5889999999999998E-2</v>
-      </c>
-      <c r="F8">
-        <v>1000</v>
+        <v>1.1283E-2</v>
+      </c>
+      <c r="F8" s="21">
+        <v>4550</v>
       </c>
       <c r="G8">
-        <v>10773</v>
+        <v>11965</v>
       </c>
       <c r="H8" s="19">
-        <v>5.479307489268239E-6</v>
+        <v>8.2792149103148756E-6</v>
       </c>
       <c r="I8" s="19">
-        <v>1.9735515242487768E-5</v>
-      </c>
-      <c r="J8">
-        <v>7.6189999999999994E-2</v>
-      </c>
-      <c r="K8" s="18">
-        <v>3</v>
-      </c>
-      <c r="L8" s="18">
-        <f t="shared" si="0"/>
-        <v>0.97500000000000009</v>
+        <v>2.1695450437220412E-5</v>
+      </c>
+      <c r="J8" s="16">
+        <v>0.377</v>
+      </c>
+      <c r="K8" s="16">
+        <v>4.4621380803155093</v>
+      </c>
+      <c r="L8" s="16">
+        <v>1.4374449171319685</v>
       </c>
       <c r="M8" s="16">
-        <f t="shared" si="2"/>
-        <v>3.4499999999999997</v>
+        <v>9.2447120071420521</v>
       </c>
       <c r="N8" s="16">
-        <f t="shared" si="1"/>
-        <v>0.96599999999999997</v>
+        <v>2.6789344608879491</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" t="s">
         <v>91</v>
       </c>
-      <c r="B9" t="s">
-        <v>92</v>
-      </c>
-      <c r="C9" s="2">
-        <v>46167.178819444445</v>
-      </c>
-      <c r="D9">
-        <v>7.2220000000000004</v>
+      <c r="C9" s="20">
+        <v>44803</v>
+      </c>
+      <c r="D9" s="16">
+        <v>19.643999999999998</v>
       </c>
       <c r="E9" s="18">
-        <v>2.324E-2</v>
-      </c>
-      <c r="F9">
-        <v>932</v>
+        <v>1.0130999999999999E-2</v>
+      </c>
+      <c r="F9" s="21">
+        <v>4300</v>
       </c>
       <c r="G9">
-        <v>10632</v>
+        <v>11525</v>
       </c>
       <c r="H9" s="19">
-        <v>5.5397125284684755E-6</v>
+        <v>8.6366298691718819E-6</v>
       </c>
       <c r="I9" s="19">
-        <v>1.9777798769927931E-5</v>
-      </c>
-      <c r="J9">
-        <v>0.10365000000000001</v>
-      </c>
-      <c r="K9" s="18">
-        <v>3.2</v>
-      </c>
-      <c r="L9" s="18">
-        <f t="shared" si="0"/>
-        <v>1.04</v>
+        <v>2.1945640908420317E-5</v>
+      </c>
+      <c r="J9" s="16">
+        <v>0.48899999999999999</v>
+      </c>
+      <c r="K9" s="16">
+        <v>4.9867925005573994</v>
+      </c>
+      <c r="L9" s="16">
+        <v>1.6265974731023589</v>
       </c>
       <c r="M9" s="16">
-        <f t="shared" si="2"/>
-        <v>3.6799999999999997</v>
+        <v>10.463479944997566</v>
       </c>
       <c r="N9" s="16">
-        <f t="shared" si="1"/>
-        <v>1.0304</v>
+        <v>3.0117804927713299</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" t="s">
         <v>93</v>
       </c>
-      <c r="B10" t="s">
-        <v>94</v>
-      </c>
-      <c r="C10" s="2">
-        <v>46243.127280092594</v>
-      </c>
-      <c r="D10">
-        <v>4.9690000000000003</v>
+      <c r="C10" s="20">
+        <v>44818</v>
+      </c>
+      <c r="D10" s="16">
+        <v>15.125999999999999</v>
       </c>
       <c r="E10" s="18">
-        <v>3.6600000000000001E-2</v>
-      </c>
-      <c r="F10">
-        <v>735</v>
+        <v>9.2700000000000005E-3</v>
+      </c>
+      <c r="F10" s="21">
+        <v>4130</v>
       </c>
       <c r="G10">
-        <v>10335</v>
+        <v>11330</v>
       </c>
       <c r="H10" s="19">
-        <v>5.6738879694443745E-6</v>
+        <v>8.8070898565790042E-6</v>
       </c>
       <c r="I10" s="19">
-        <v>1.9871721578611061E-5</v>
-      </c>
-      <c r="J10">
-        <v>0.15081</v>
-      </c>
-      <c r="K10" s="18">
-        <v>3.54</v>
-      </c>
-      <c r="L10" s="18">
-        <f t="shared" si="0"/>
-        <v>1.1505000000000001</v>
+        <v>2.2064962899605303E-5</v>
+      </c>
+      <c r="J10" s="16">
+        <v>0.55800000000000005</v>
+      </c>
+      <c r="K10" s="16">
+        <v>5.4469665324725387</v>
+      </c>
+      <c r="L10" s="16">
+        <v>1.7802222222222224</v>
       </c>
       <c r="M10" s="16">
-        <f t="shared" si="2"/>
-        <v>4.0709999999999997</v>
+        <v>12.932360213695913</v>
       </c>
       <c r="N10" s="16">
-        <f t="shared" si="1"/>
-        <v>1.13988</v>
+        <v>3.6515409229141875</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>95</v>
-      </c>
-      <c r="C11" s="2">
-        <v>46093.428402777776</v>
-      </c>
-      <c r="D11" s="16"/>
-      <c r="E11">
-        <v>3.8359999999999998E-2</v>
-      </c>
-      <c r="F11" s="22" t="e">
-        <v>#REF!</v>
+        <v>94</v>
+      </c>
+      <c r="C11" s="20">
+        <v>44831</v>
+      </c>
+      <c r="D11" s="16">
+        <v>15.686999999999999</v>
+      </c>
+      <c r="E11" s="18">
+        <v>8.933E-3</v>
+      </c>
+      <c r="F11" s="21">
+        <v>4075</v>
       </c>
       <c r="G11">
-        <v>10457</v>
+        <v>11142</v>
       </c>
       <c r="H11" s="19">
-        <v>5.6175724188731071E-6</v>
+        <v>8.9792279149939014E-6</v>
       </c>
       <c r="I11" s="19">
-        <v>1.9832300693211174E-5</v>
-      </c>
-      <c r="J11">
-        <v>2.1508099999999999</v>
-      </c>
-      <c r="K11" s="18">
-        <v>4</v>
-      </c>
-      <c r="L11" s="18">
-        <f t="shared" si="0"/>
-        <v>1.3</v>
+        <v>2.2185459540495729E-5</v>
+      </c>
+      <c r="J11" s="16">
+        <v>0.61599999999999999</v>
+      </c>
+      <c r="K11" s="16">
+        <v>5.6618488513973206</v>
+      </c>
+      <c r="L11" s="16">
+        <v>1.8632853464681518</v>
       </c>
       <c r="M11" s="16">
-        <f t="shared" si="2"/>
-        <v>4.5999999999999996</v>
+        <v>12.324986022970865</v>
       </c>
       <c r="N11" s="16">
-        <f t="shared" si="1"/>
-        <v>1.288</v>
+        <v>3.5103488238668965</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>96</v>
-      </c>
-      <c r="C12" s="2">
-        <v>46101.53</v>
-      </c>
-      <c r="D12" s="16"/>
-      <c r="E12">
-        <v>1.4924E-2</v>
-      </c>
-      <c r="F12" s="22" t="e">
-        <v>#REF!</v>
+        <v>95</v>
+      </c>
+      <c r="C12" s="20">
+        <v>44833</v>
+      </c>
+      <c r="D12" s="16">
+        <v>13.723000000000001</v>
+      </c>
+      <c r="E12" s="18">
+        <v>5.3169999999999997E-3</v>
+      </c>
+      <c r="F12" s="21">
+        <v>4055</v>
       </c>
       <c r="G12">
-        <v>10367</v>
+        <v>11122</v>
       </c>
       <c r="H12" s="19">
-        <v>5.6589479624400542E-6</v>
+        <v>8.9980131360874166E-6</v>
       </c>
       <c r="I12" s="19">
-        <v>1.9861263573708037E-5</v>
-      </c>
-      <c r="J12">
-        <v>3.1508099999999999</v>
-      </c>
-      <c r="K12" s="18">
-        <v>5.5</v>
-      </c>
-      <c r="L12" s="18">
-        <f t="shared" si="0"/>
-        <v>1.7875000000000001</v>
+        <v>2.2198609195261192E-5</v>
+      </c>
+      <c r="J12" s="16">
+        <v>0.63</v>
+      </c>
+      <c r="K12" s="16">
+        <v>9.1024219000692526</v>
+      </c>
+      <c r="L12" s="16">
+        <v>2.7217810795561408</v>
       </c>
       <c r="M12" s="16">
-        <f t="shared" si="2"/>
-        <v>6.3249999999999993</v>
+        <v>13.941163861329127</v>
       </c>
       <c r="N12" s="16">
-        <f t="shared" si="1"/>
-        <v>1.7709999999999999</v>
+        <v>3.9164322669970124</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>97</v>
-      </c>
-      <c r="C13" s="2">
-        <v>46106.668703703705</v>
-      </c>
-      <c r="D13" s="16"/>
-      <c r="E13">
-        <v>7.4020000000000002E-2</v>
-      </c>
-      <c r="F13" s="22" t="e">
-        <v>#REF!</v>
+        <v>96</v>
+      </c>
+      <c r="C13" s="20">
+        <v>44846</v>
+      </c>
+      <c r="D13" s="16">
+        <v>11.512</v>
+      </c>
+      <c r="E13" s="18">
+        <v>8.7840000000000001E-3</v>
+      </c>
+      <c r="F13" s="21">
+        <v>3945</v>
       </c>
       <c r="G13">
-        <v>10328</v>
+        <v>10979</v>
       </c>
       <c r="H13" s="19">
-        <v>5.6771724062387215E-6</v>
+        <v>9.1350841146718146E-6</v>
       </c>
       <c r="I13" s="19">
-        <v>1.9874020684367105E-5</v>
-      </c>
-      <c r="J13">
-        <v>4.1508099999999999</v>
-      </c>
-      <c r="K13" s="18">
-        <v>6</v>
-      </c>
-      <c r="L13" s="18">
-        <f t="shared" si="0"/>
-        <v>1.9500000000000002</v>
+        <v>2.2294558880270269E-5</v>
+      </c>
+      <c r="J13" s="16">
+        <v>0.67800000000000005</v>
+      </c>
+      <c r="K13" s="16">
+        <v>5.7843289549548373</v>
+      </c>
+      <c r="L13" s="16">
+        <v>1.927886156648452</v>
       </c>
       <c r="M13" s="16">
-        <f t="shared" si="2"/>
-        <v>6.8999999999999995</v>
+        <v>16.048830830140322</v>
       </c>
       <c r="N13" s="16">
-        <f t="shared" si="1"/>
-        <v>1.9319999999999999</v>
+        <v>4.4403484190410012</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C14" s="2">
-        <v>46118.550451388888</v>
-      </c>
-      <c r="D14" s="16"/>
-      <c r="E14">
-        <v>1.2886E-2</v>
-      </c>
-      <c r="F14" s="22" t="e">
-        <v>#REF!</v>
+        <v>87</v>
+      </c>
+      <c r="C14" s="20">
+        <v>44857</v>
+      </c>
+      <c r="D14" s="16">
+        <v>11.023999999999999</v>
+      </c>
+      <c r="E14" s="18">
+        <v>1.3225000000000001E-2</v>
+      </c>
+      <c r="F14" s="21">
+        <v>3880</v>
       </c>
       <c r="G14">
-        <v>10228</v>
+        <v>10883</v>
       </c>
       <c r="H14" s="19">
-        <v>5.7247456065667185E-6</v>
+        <v>9.2298959105538258E-6</v>
       </c>
       <c r="I14" s="19">
-        <v>1.9907321924596702E-5</v>
-      </c>
-      <c r="J14">
-        <v>5.1508099999999999</v>
-      </c>
-      <c r="K14" s="18">
-        <v>8.25</v>
-      </c>
-      <c r="L14" s="18">
-        <f t="shared" si="0"/>
-        <v>2.6812499999999999</v>
+        <v>2.2360927137387679E-5</v>
+      </c>
+      <c r="J14" s="16">
+        <v>0.72845860920204608</v>
+      </c>
+      <c r="K14" s="16">
+        <v>4.1099984829781517</v>
+      </c>
+      <c r="L14" s="16">
+        <v>1.5513697623211387</v>
       </c>
       <c r="M14" s="16">
-        <f t="shared" si="2"/>
-        <v>9.4874999999999989</v>
+        <v>16.468385635968495</v>
       </c>
       <c r="N14" s="16">
-        <f t="shared" si="1"/>
-        <v>2.6564999999999999</v>
+        <v>4.5588323392455878</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>98</v>
-      </c>
-      <c r="C15" s="2">
-        <v>46125.371180555558</v>
-      </c>
-      <c r="D15" s="16"/>
-      <c r="E15">
-        <v>1.7957999999999998E-2</v>
-      </c>
-      <c r="F15" s="22" t="e">
-        <v>#REF!</v>
+        <v>97</v>
+      </c>
+      <c r="C15" s="20">
+        <v>44877</v>
+      </c>
+      <c r="D15" s="16">
+        <v>10.749000000000001</v>
+      </c>
+      <c r="E15" s="18">
+        <v>9.4940000000000007E-3</v>
+      </c>
+      <c r="F15" s="21">
+        <v>3775</v>
       </c>
       <c r="G15">
-        <v>10167</v>
+        <v>10652</v>
       </c>
       <c r="H15" s="19">
-        <v>5.7543791906410511E-6</v>
+        <v>9.4676989011167314E-6</v>
       </c>
       <c r="I15" s="19">
-        <v>1.9928065433448735E-5</v>
-      </c>
-      <c r="J15">
-        <v>6.1508099999999999</v>
-      </c>
-      <c r="K15" s="18">
-        <v>9.36</v>
-      </c>
-      <c r="L15" s="18">
-        <f t="shared" si="0"/>
-        <v>3.0419999999999998</v>
+        <v>2.2527389230781713E-5</v>
+      </c>
+      <c r="J15" s="16">
+        <v>0.81045860920204604</v>
+      </c>
+      <c r="K15" s="16">
+        <v>5.4860861675183381</v>
+      </c>
+      <c r="L15" s="16">
+        <v>1.9324303808472956</v>
       </c>
       <c r="M15" s="16">
-        <f t="shared" si="2"/>
-        <v>10.763999999999999</v>
+        <v>16.40016838182482</v>
       </c>
       <c r="N15" s="16">
-        <f t="shared" si="1"/>
-        <v>3.0139200000000002</v>
+        <v>4.5513926495778945</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>99</v>
-      </c>
-      <c r="C16" s="2">
-        <v>46131.612326388888</v>
-      </c>
-      <c r="D16" s="16"/>
-      <c r="E16">
-        <v>3.9039999999999998E-2</v>
-      </c>
-      <c r="F16" s="22" t="e">
-        <v>#REF!</v>
+        <v>98</v>
+      </c>
+      <c r="C16" s="20">
+        <v>44885</v>
+      </c>
+      <c r="D16" s="16">
+        <v>7.4909999999999997</v>
+      </c>
+      <c r="E16" s="18">
+        <v>1.6306999999999999E-2</v>
+      </c>
+      <c r="F16" s="21">
+        <v>3720</v>
       </c>
       <c r="G16">
-        <v>10104</v>
+        <v>9742</v>
       </c>
       <c r="H16" s="19">
-        <v>5.7854884878310361E-6</v>
+        <v>1.0554307442604296E-5</v>
       </c>
       <c r="I16" s="19">
-        <v>1.9949841941481724E-5</v>
-      </c>
-      <c r="J16">
-        <v>7.1508099999999999</v>
-      </c>
-      <c r="K16" s="18">
-        <v>11.525</v>
-      </c>
-      <c r="L16" s="18">
-        <f t="shared" si="0"/>
-        <v>3.7456250000000004</v>
+        <v>2.3288015209823009E-5</v>
+      </c>
+      <c r="J16" s="16">
+        <v>0.84445860920204607</v>
+      </c>
+      <c r="K16" s="16">
+        <v>3.4777168544655259</v>
+      </c>
+      <c r="L16" s="16">
+        <v>1.441870763491615</v>
       </c>
       <c r="M16" s="16">
-        <f t="shared" si="2"/>
-        <v>13.25375</v>
+        <v>22.168556460557404</v>
       </c>
       <c r="N16" s="16">
-        <f t="shared" si="1"/>
-        <v>3.7110500000000002</v>
+        <v>5.6822960140879086</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="2">
-        <v>46141.80296296296</v>
-      </c>
-      <c r="D17" s="16"/>
-      <c r="E17">
-        <v>2.4459999999999999E-2</v>
-      </c>
-      <c r="F17" s="22" t="e">
-        <v>#REF!</v>
+        <v>89</v>
+      </c>
+      <c r="C17" s="20">
+        <v>44899</v>
+      </c>
+      <c r="D17" s="16">
+        <v>6.4720000000000004</v>
+      </c>
+      <c r="E17" s="18">
+        <v>1.2567999999999999E-2</v>
+      </c>
+      <c r="F17" s="21">
+        <v>3675</v>
       </c>
       <c r="G17">
-        <v>10029</v>
+        <v>9599</v>
       </c>
       <c r="H17" s="19">
-        <v>5.8232098343631589E-6</v>
+        <v>1.0749344484912831E-5</v>
       </c>
       <c r="I17" s="19">
-        <v>1.9976246884054212E-5</v>
-      </c>
-      <c r="J17">
-        <v>8.1508099999999999</v>
-      </c>
-      <c r="K17" s="18">
-        <v>12</v>
-      </c>
-      <c r="L17" s="18">
-        <f>K17*0.325</f>
-        <v>3.9000000000000004</v>
+        <v>2.3424541139438982E-5</v>
+      </c>
+      <c r="J17" s="16">
+        <v>0.86845860920204609</v>
+      </c>
+      <c r="K17" s="16">
+        <v>4.2652019735612567</v>
+      </c>
+      <c r="L17" s="16">
+        <v>1.632223726961435</v>
       </c>
       <c r="M17" s="16">
-        <f t="shared" si="2"/>
-        <v>13.799999999999999</v>
+        <v>25.109302933522905</v>
       </c>
       <c r="N17" s="16">
-        <f>M17*0.28</f>
-        <v>3.8639999999999999</v>
+        <v>6.3190650677928986</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C18" s="21"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="22"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="16"/>
+      <c r="C18" s="20">
+        <v>44915</v>
+      </c>
+      <c r="D18" s="16">
+        <v>10.425000000000001</v>
+      </c>
+      <c r="E18" s="18">
+        <v>1.515E-2</v>
+      </c>
+      <c r="F18" s="21">
+        <v>3780</v>
+      </c>
+      <c r="G18">
+        <v>9475</v>
+      </c>
+      <c r="H18" s="19">
+        <v>1.0924322593953131E-5</v>
+      </c>
+      <c r="I18" s="19">
+        <v>2.3547025815767191E-5</v>
+      </c>
+      <c r="J18" s="16">
+        <v>0.91500000000000004</v>
+      </c>
+      <c r="K18" s="16">
+        <v>3.718182073885004</v>
+      </c>
+      <c r="L18" s="16">
+        <v>1.5404125412541254</v>
+      </c>
+      <c r="M18" s="16">
+        <v>16.313544635508155</v>
+      </c>
+      <c r="N18" s="16">
+        <v>4.3505395683453241</v>
+      </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C19" s="21"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="22"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="16"/>
+      <c r="C19" s="20">
+        <v>44932</v>
+      </c>
+      <c r="D19" s="16">
+        <v>7.5350000000000001</v>
+      </c>
+      <c r="E19" s="18">
+        <v>1.4071999999999999E-2</v>
+      </c>
+      <c r="F19" s="21">
+        <v>3670</v>
+      </c>
+      <c r="G19">
+        <v>9392</v>
+      </c>
+      <c r="H19" s="19">
+        <v>1.1044563035856902E-5</v>
+      </c>
+      <c r="I19" s="19">
+        <v>2.3631194125099829E-5</v>
+      </c>
+      <c r="J19" s="16">
+        <v>0.97699999999999998</v>
+      </c>
+      <c r="K19" s="16">
+        <v>3.9841736392239597</v>
+      </c>
+      <c r="L19" s="16">
+        <v>1.6444246731097214</v>
+      </c>
+      <c r="M19" s="16">
+        <v>21.587908712110895</v>
+      </c>
+      <c r="N19" s="16">
+        <v>5.5514711347047117</v>
+      </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C20" s="21"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="22"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="16"/>
+      <c r="C20" s="20">
+        <v>44944</v>
+      </c>
+      <c r="D20" s="16">
+        <v>7.2720000000000002</v>
+      </c>
+      <c r="E20" s="18">
+        <v>2.1100000000000001E-2</v>
+      </c>
+      <c r="F20" s="21">
+        <v>3570</v>
+      </c>
+      <c r="G20">
+        <v>9330</v>
+      </c>
+      <c r="H20" s="19">
+        <v>1.1136044698779005E-5</v>
+      </c>
+      <c r="I20" s="19">
+        <v>2.3695231289145303E-5</v>
+      </c>
+      <c r="J20" s="16">
+        <v>1.02</v>
+      </c>
+      <c r="K20" s="16">
+        <v>3.0201224866971721</v>
+      </c>
+      <c r="L20" s="16">
+        <v>1.4621800947867298</v>
+      </c>
+      <c r="M20" s="16">
+        <v>21.738265477920507</v>
+      </c>
+      <c r="N20" s="16">
+        <v>5.6003217821782183</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C21" s="21"/>
-      <c r="D21" s="16"/>
-      <c r="F21" s="22"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="16"/>
+      <c r="C21" s="20">
+        <v>44965</v>
+      </c>
+      <c r="D21" s="16">
+        <v>7.3070000000000004</v>
+      </c>
+      <c r="E21" s="18">
+        <v>1.2446E-2</v>
+      </c>
+      <c r="F21" s="21">
+        <v>3440</v>
+      </c>
+      <c r="G21">
+        <v>9212</v>
+      </c>
+      <c r="H21" s="19">
+        <v>1.1314159112058182E-5</v>
+      </c>
+      <c r="I21" s="19">
+        <v>2.3819911378440726E-5</v>
+      </c>
+      <c r="J21" s="16">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="K21" s="16">
+        <v>4.4631065658972542</v>
+      </c>
+      <c r="L21" s="16">
+        <v>1.8301574803149607</v>
+      </c>
+      <c r="M21" s="16">
+        <v>20.854197900355942</v>
+      </c>
+      <c r="N21" s="16">
+        <v>5.4268386478719028</v>
+      </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C22" s="15"/>
-      <c r="D22" s="16"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="16"/>
+      <c r="C22" s="20">
+        <v>45003</v>
+      </c>
+      <c r="D22" s="16">
+        <v>8.657</v>
+      </c>
+      <c r="E22" s="18">
+        <v>1.6556999999999999E-2</v>
+      </c>
+      <c r="F22" s="21">
+        <v>3180</v>
+      </c>
+      <c r="G22">
+        <v>9200</v>
+      </c>
+      <c r="H22" s="19">
+        <v>1.1332570496000007E-5</v>
+      </c>
+      <c r="I22" s="19">
+        <v>2.3832799347200005E-5</v>
+      </c>
+      <c r="J22" s="16">
+        <v>1.182714</v>
+      </c>
+      <c r="K22" s="16">
+        <v>3.7169280514322001</v>
+      </c>
+      <c r="L22" s="16">
+        <v>1.7383702179138734</v>
+      </c>
+      <c r="M22" s="16">
+        <v>16.595624121013064</v>
+      </c>
+      <c r="N22" s="16">
+        <v>4.5621757072888993</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C23" s="15"/>
-      <c r="D23" s="16"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="K23" s="18"/>
-      <c r="L23" s="18"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="16"/>
+      <c r="C23" s="20">
+        <v>45039</v>
+      </c>
+      <c r="D23" s="16">
+        <v>2.66</v>
+      </c>
+      <c r="E23" s="18">
+        <v>1.9E-2</v>
+      </c>
+      <c r="F23" s="21">
+        <v>2720</v>
+      </c>
+      <c r="G23">
+        <v>9093</v>
+      </c>
+      <c r="H23" s="19">
+        <v>1.149921137141482E-5</v>
+      </c>
+      <c r="I23" s="19">
+        <v>2.3949447959990374E-5</v>
+      </c>
+      <c r="J23" s="16">
+        <v>1.28</v>
+      </c>
+      <c r="K23" s="16">
+        <v>3.4776113618691351</v>
+      </c>
+      <c r="L23" s="16">
+        <v>1.758578947368421</v>
+      </c>
+      <c r="M23" s="16">
+        <v>43.976449316314621</v>
+      </c>
+      <c r="N23" s="16">
+        <v>10.578105263157894</v>
+      </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C24" s="15"/>
-      <c r="D24" s="16"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="16"/>
+      <c r="C24" s="20">
+        <v>45059</v>
+      </c>
+      <c r="D24" s="16">
+        <v>2.34</v>
+      </c>
+      <c r="E24" s="18">
+        <v>1.6660000000000001E-2</v>
+      </c>
+      <c r="F24" s="21">
+        <v>2550</v>
+      </c>
+      <c r="G24">
+        <v>8997</v>
+      </c>
+      <c r="H24" s="19">
+        <v>1.1652560885268289E-5</v>
+      </c>
+      <c r="I24" s="19">
+        <v>2.4056792619687801E-5</v>
+      </c>
+      <c r="J24" s="16">
+        <v>1.3380000000000001</v>
+      </c>
+      <c r="K24" s="16">
+        <v>3.833096106648838</v>
+      </c>
+      <c r="L24" s="16">
+        <v>1.8780360144057624</v>
+      </c>
+      <c r="M24" s="16">
+        <v>46.636789700325899</v>
+      </c>
+      <c r="N24" s="16">
+        <v>11.142423076923077</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C25" s="15"/>
-      <c r="D25" s="16"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="K25" s="18"/>
-      <c r="L25" s="18"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="16"/>
+      <c r="C25" s="20">
+        <v>45085</v>
+      </c>
+      <c r="D25" s="16">
+        <v>6.09</v>
+      </c>
+      <c r="E25">
+        <v>1.7493999999999999E-2</v>
+      </c>
+      <c r="F25" s="21">
+        <v>2420</v>
+      </c>
+      <c r="G25">
+        <v>8975</v>
+      </c>
+      <c r="H25" s="19">
+        <v>1.1688222731140632E-5</v>
+      </c>
+      <c r="I25" s="19">
+        <v>2.4081755911798442E-5</v>
+      </c>
+      <c r="J25" s="16">
+        <v>1.397</v>
+      </c>
+      <c r="K25" s="16">
+        <v>3.7706830448933779</v>
+      </c>
+      <c r="L25" s="16">
+        <v>1.9100330398993941</v>
+      </c>
+      <c r="M25" s="16">
+        <v>17.897987039970889</v>
+      </c>
+      <c r="N25" s="16">
+        <v>4.9634203612479473</v>
+      </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C26" s="15"/>
-      <c r="D26" s="16"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
-      <c r="K26" s="18"/>
-      <c r="L26" s="18"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="16"/>
+      <c r="C26" s="15">
+        <v>45104</v>
+      </c>
+      <c r="D26" s="16">
+        <v>4.8959999999999999</v>
+      </c>
+      <c r="E26">
+        <v>8.0700000000000008E-3</v>
+      </c>
+      <c r="F26">
+        <v>2300</v>
+      </c>
+      <c r="G26">
+        <v>8900</v>
+      </c>
+      <c r="H26" s="19">
+        <v>1.1811270923000008E-5</v>
+      </c>
+      <c r="I26" s="19">
+        <v>2.4167889646100008E-5</v>
+      </c>
+      <c r="J26" s="16">
+        <v>1.4470000000000001</v>
+      </c>
+      <c r="K26" s="16">
+        <v>6.5742882785044205</v>
+      </c>
+      <c r="L26" s="16">
+        <v>2.5498500619578683</v>
+      </c>
+      <c r="M26" s="16">
+        <v>20.88482633523704</v>
+      </c>
+      <c r="N26" s="16">
+        <v>5.6279640522875818</v>
+      </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C27" s="21"/>
-      <c r="D27" s="16"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
-      <c r="K27" s="18"/>
-      <c r="L27" s="18"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="16"/>
+      <c r="C27" s="15">
+        <v>45114</v>
+      </c>
+      <c r="D27" s="16">
+        <v>0.93100000000000005</v>
+      </c>
+      <c r="E27">
+        <v>4.2199999999999998E-3</v>
+      </c>
+      <c r="F27">
+        <v>2276</v>
+      </c>
+      <c r="G27">
+        <v>8791</v>
+      </c>
+      <c r="H27" s="19">
+        <v>1.1994218435009664E-5</v>
+      </c>
+      <c r="I27" s="19">
+        <v>2.4295952904506763E-5</v>
+      </c>
+      <c r="J27" s="16">
+        <v>1.4697</v>
+      </c>
+      <c r="K27" s="16">
+        <v>11.223045570594754</v>
+      </c>
+      <c r="L27" s="16">
+        <v>3.552875355450237</v>
+      </c>
+      <c r="M27" s="16">
+        <v>102.09070243695257</v>
+      </c>
+      <c r="N27" s="16">
+        <v>22.960909452201932</v>
+      </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C28" s="21"/>
-      <c r="D28" s="16"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="K28" s="18"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="16"/>
+      <c r="C28" s="15">
+        <v>45122</v>
+      </c>
+      <c r="D28" s="16">
+        <v>1.5112000000000001</v>
+      </c>
+      <c r="E28">
+        <v>1.0331999999999999E-2</v>
+      </c>
+      <c r="F28">
+        <v>2241</v>
+      </c>
+      <c r="G28">
+        <v>8728</v>
+      </c>
+      <c r="H28" s="19">
+        <v>1.2102218776169991E-5</v>
+      </c>
+      <c r="I28" s="19">
+        <v>2.4371553143318991E-5</v>
+      </c>
+      <c r="J28" s="16">
+        <v>1.4887999999999999</v>
+      </c>
+      <c r="K28" s="16">
+        <v>5.4600972572315563</v>
+      </c>
+      <c r="L28" s="16">
+        <v>2.3335541618273323</v>
+      </c>
+      <c r="M28" s="16">
+        <v>62.335454545729569</v>
+      </c>
+      <c r="N28" s="16">
+        <v>14.43179100052938</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C29" s="21"/>
-      <c r="D29" s="16"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="19"/>
-      <c r="K29" s="18"/>
-      <c r="L29" s="18"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="16"/>
+      <c r="C29" s="15">
+        <v>45151</v>
+      </c>
+      <c r="D29" s="16">
+        <v>1.7686999999999999</v>
+      </c>
+      <c r="E29">
+        <v>1.2028E-2</v>
+      </c>
+      <c r="F29">
+        <v>2095</v>
+      </c>
+      <c r="G29">
+        <v>8610</v>
+      </c>
+      <c r="H29" s="19">
+        <v>1.2309041674227002E-5</v>
+      </c>
+      <c r="I29" s="19">
+        <v>2.4516329171958903E-5</v>
+      </c>
+      <c r="J29" s="16">
+        <v>1.5504</v>
+      </c>
+      <c r="K29" s="16">
+        <v>4.9415822994899052</v>
+      </c>
+      <c r="L29" s="16">
+        <v>2.2662297306285333</v>
+      </c>
+      <c r="M29" s="16">
+        <v>49.864557156592014</v>
+      </c>
+      <c r="N29" s="16">
+        <v>11.748822570249336</v>
+      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C30" s="21"/>
-      <c r="D30" s="16"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
-      <c r="K30" s="18"/>
-      <c r="L30" s="18"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="16"/>
+      <c r="C30" s="15">
+        <v>45162</v>
+      </c>
+      <c r="D30" s="16">
+        <v>7.13</v>
+      </c>
+      <c r="E30">
+        <v>1.4749999999999999E-2</v>
+      </c>
+      <c r="F30">
+        <v>2045</v>
+      </c>
+      <c r="G30">
+        <v>8561</v>
+      </c>
+      <c r="H30" s="19">
+        <v>1.2396688774358935E-5</v>
+      </c>
+      <c r="I30" s="19">
+        <v>2.4577682142051255E-5</v>
+      </c>
+      <c r="J30" s="16">
+        <v>1.5723</v>
+      </c>
+      <c r="K30" s="16">
+        <v>4.3307623227547865</v>
+      </c>
+      <c r="L30" s="16">
+        <v>2.1527067796610169</v>
+      </c>
+      <c r="M30" s="16">
+        <v>13.242085117530809</v>
+      </c>
+      <c r="N30" s="16">
+        <v>4.0277340813464235</v>
+      </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C31" s="21"/>
-      <c r="D31" s="16"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="19"/>
-      <c r="K31" s="18"/>
-      <c r="L31" s="18"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="16"/>
+      <c r="C31" s="20">
+        <v>45168</v>
+      </c>
+      <c r="D31" s="16">
+        <v>6.75</v>
+      </c>
+      <c r="E31">
+        <v>1.5538E-2</v>
+      </c>
+      <c r="F31">
+        <v>2010</v>
+      </c>
+      <c r="G31">
+        <v>8532</v>
+      </c>
+      <c r="H31" s="19">
+        <v>1.2449054759365061E-5</v>
+      </c>
+      <c r="I31" s="19">
+        <v>2.4614338331555543E-5</v>
+      </c>
+      <c r="J31" s="16">
+        <v>1.5825</v>
+      </c>
+      <c r="K31" s="16">
+        <v>4.1971689953934135</v>
+      </c>
+      <c r="L31" s="16">
+        <v>2.1316054189728408</v>
+      </c>
+      <c r="M31" s="16">
+        <v>13.680236439903693</v>
+      </c>
+      <c r="N31" s="16">
+        <v>4.1231399999999994</v>
+      </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C32" s="21"/>
-      <c r="D32" s="16"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="19"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="16"/>
+      <c r="C32" s="20">
+        <v>45181</v>
+      </c>
+      <c r="D32" s="16">
+        <v>2.21</v>
+      </c>
+      <c r="E32">
+        <v>1.6326E-2</v>
+      </c>
+      <c r="F32">
+        <v>1927</v>
+      </c>
+      <c r="G32">
+        <v>8500</v>
+      </c>
+      <c r="H32" s="19">
+        <v>1.2507266374999995E-5</v>
+      </c>
+      <c r="I32" s="19">
+        <v>2.4655086462499995E-5</v>
+      </c>
+      <c r="J32" s="16">
+        <v>1.6111899999999999</v>
+      </c>
+      <c r="K32" s="16">
+        <v>4.0955451363269697</v>
+      </c>
+      <c r="L32" s="16">
+        <v>2.1318319208624281</v>
+      </c>
+      <c r="M32" s="16">
+        <v>36.976943135105891</v>
+      </c>
+      <c r="N32" s="16">
+        <v>9.0227284615384615</v>
+      </c>
     </row>
     <row r="33" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C33" s="21"/>
-      <c r="D33" s="16"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="K33" s="18"/>
-      <c r="L33" s="18"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="16"/>
+      <c r="C33" s="20">
+        <v>45204</v>
+      </c>
+      <c r="D33" s="16">
+        <v>2.8660000000000001</v>
+      </c>
+      <c r="E33">
+        <v>1.0828000000000001E-2</v>
+      </c>
+      <c r="F33">
+        <v>1840</v>
+      </c>
+      <c r="G33">
+        <v>8498</v>
+      </c>
+      <c r="H33" s="19">
+        <v>1.2510919583519872E-5</v>
+      </c>
+      <c r="I33" s="19">
+        <v>2.465764370846391E-5</v>
+      </c>
+      <c r="J33" s="16">
+        <v>1.65398</v>
+      </c>
+      <c r="K33" s="16">
+        <v>5.399397022402634</v>
+      </c>
+      <c r="L33" s="16">
+        <v>2.4387971407462135</v>
+      </c>
+      <c r="M33" s="16">
+        <v>27.690927297341009</v>
+      </c>
+      <c r="N33" s="16">
+        <v>7.1097790230286106</v>
+      </c>
     </row>
     <row r="34" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C34" s="21"/>
-      <c r="D34" s="16"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19"/>
-      <c r="K34" s="18"/>
-      <c r="L34" s="18"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="16"/>
+      <c r="C34" s="20">
+        <v>45215</v>
+      </c>
+      <c r="D34" s="16">
+        <v>3.9860000000000002</v>
+      </c>
+      <c r="E34">
+        <v>1.1244000000000001E-2</v>
+      </c>
+      <c r="F34">
+        <v>1835</v>
+      </c>
+      <c r="G34">
+        <v>8611</v>
+      </c>
+      <c r="H34" s="19">
+        <v>1.230726380773748E-5</v>
+      </c>
+      <c r="I34" s="19">
+        <v>2.4515084665416237E-5</v>
+      </c>
+      <c r="J34" s="16">
+        <v>1.67466</v>
+      </c>
+      <c r="K34" s="16">
+        <v>5.3024802913654447</v>
+      </c>
+      <c r="L34" s="16">
+        <v>2.4404906652436855</v>
+      </c>
+      <c r="M34" s="16">
+        <v>20.453353637347583</v>
+      </c>
+      <c r="N34" s="16">
+        <v>5.6388308479678875</v>
+      </c>
     </row>
     <row r="35" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C35" s="21"/>
-      <c r="D35" s="16"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="19"/>
-      <c r="K35" s="18"/>
-      <c r="L35" s="18"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="16"/>
+      <c r="C35" s="20">
+        <v>45221</v>
+      </c>
+      <c r="D35" s="16">
+        <v>9.5299999999999994</v>
+      </c>
+      <c r="E35">
+        <v>9.6360000000000005E-3</v>
+      </c>
+      <c r="F35">
+        <v>1785</v>
+      </c>
+      <c r="G35">
+        <v>8455</v>
+      </c>
+      <c r="H35" s="19">
+        <v>1.2589891879819626E-5</v>
+      </c>
+      <c r="I35" s="19">
+        <v>2.4712924315873735E-5</v>
+      </c>
+      <c r="J35" s="16">
+        <v>1.6836599999999999</v>
+      </c>
+      <c r="K35" s="16">
+        <v>5.8829809589978028</v>
+      </c>
+      <c r="L35" s="16">
+        <v>2.5610987712743878</v>
+      </c>
+      <c r="M35" s="16">
+        <v>9.2628218382173717</v>
+      </c>
+      <c r="N35" s="16">
+        <v>3.2673090031479539</v>
+      </c>
     </row>
     <row r="36" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C36" s="21"/>
-      <c r="D36" s="16"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="19"/>
-      <c r="K36" s="18"/>
-      <c r="L36" s="18"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="16"/>
+      <c r="C36" s="20">
+        <v>45229</v>
+      </c>
+      <c r="D36" s="16">
+        <v>2.0409999999999999</v>
+      </c>
+      <c r="E36">
+        <v>9.3769999999999999E-3</v>
+      </c>
+      <c r="F36">
+        <v>1755</v>
+      </c>
+      <c r="G36">
+        <v>8413</v>
+      </c>
+      <c r="H36" s="19">
+        <v>1.2667821942236699E-5</v>
+      </c>
+      <c r="I36" s="19">
+        <v>2.4767475359565691E-5</v>
+      </c>
+      <c r="J36" s="16">
+        <v>1.6988300000000001</v>
+      </c>
+      <c r="K36" s="16">
+        <v>6.0046348677297354</v>
+      </c>
+      <c r="L36" s="16">
+        <v>2.5960252650101312</v>
+      </c>
+      <c r="M36" s="16">
+        <v>36.416644350539698</v>
+      </c>
+      <c r="N36" s="16">
+        <v>8.9329382802547777</v>
+      </c>
     </row>
     <row r="37" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C37" s="21"/>
-      <c r="D37" s="16"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="19"/>
-      <c r="K37" s="18"/>
-      <c r="L37" s="18"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="16"/>
+      <c r="C37" s="20">
+        <v>45248</v>
+      </c>
+      <c r="D37" s="16">
+        <v>4.7130000000000001</v>
+      </c>
+      <c r="E37">
+        <v>9.2180000000000005E-3</v>
+      </c>
+      <c r="F37">
+        <v>1765</v>
+      </c>
+      <c r="G37">
+        <v>8533</v>
+      </c>
+      <c r="H37">
+        <v>1.2447242902032172E-5</v>
+      </c>
+      <c r="I37" s="19">
+        <v>2.4613070031422518E-5</v>
+      </c>
+      <c r="J37" s="16">
+        <v>1.7322310000000001</v>
+      </c>
+      <c r="K37" s="16">
+        <v>6.1397836499128946</v>
+      </c>
+      <c r="L37" s="16">
+        <v>2.6579198696029507</v>
+      </c>
+      <c r="M37" s="16">
+        <v>16.9475647315878</v>
+      </c>
+      <c r="N37" s="16">
+        <v>4.9278060053044772</v>
+      </c>
     </row>
     <row r="38" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C38" s="21"/>
-      <c r="D38" s="16"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="19"/>
-      <c r="K38" s="18"/>
-      <c r="L38" s="18"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="16"/>
+      <c r="C38" s="20">
+        <v>45263</v>
+      </c>
+      <c r="D38" s="16">
+        <v>1.7794000000000001</v>
+      </c>
+      <c r="E38">
+        <v>8.09E-3</v>
+      </c>
+      <c r="F38">
+        <v>1730</v>
+      </c>
+      <c r="G38">
+        <v>8328</v>
+      </c>
+      <c r="H38">
+        <v>1.2827963735376382E-5</v>
+      </c>
+      <c r="I38" s="19">
+        <v>2.4879574614763469E-5</v>
+      </c>
+      <c r="J38" s="16">
+        <v>1.75732</v>
+      </c>
+      <c r="K38" s="16">
+        <v>6.7256281896672938</v>
+      </c>
+      <c r="L38" s="16">
+        <v>2.7867390358467246</v>
+      </c>
+      <c r="M38" s="16">
+        <v>40.835071449998068</v>
+      </c>
+      <c r="N38" s="16">
+        <v>9.854116673035854</v>
+      </c>
     </row>
     <row r="39" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C39" s="21"/>
-      <c r="D39" s="16"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
-      <c r="K39" s="18"/>
-      <c r="L39" s="18"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="16"/>
+      <c r="C39" s="20">
+        <v>45279</v>
+      </c>
+      <c r="D39" s="16">
+        <v>1.4699</v>
+      </c>
+      <c r="E39">
+        <v>8.5830000000000004E-3</v>
+      </c>
+      <c r="F39">
+        <v>1695</v>
+      </c>
+      <c r="G39">
+        <v>8292</v>
+      </c>
+      <c r="H39">
+        <v>1.2896776907426494E-5</v>
+      </c>
+      <c r="I39" s="19">
+        <v>2.4927743835198545E-5</v>
+      </c>
+      <c r="J39" s="16">
+        <v>1.7849999999999999</v>
+      </c>
+      <c r="K39" s="16">
+        <v>6.4588838370320536</v>
+      </c>
+      <c r="L39" s="16">
+        <v>2.7510957707095418</v>
+      </c>
+      <c r="M39" s="16">
+        <v>48.044287522724105</v>
+      </c>
+      <c r="N39" s="16">
+        <v>11.346834138376762</v>
+      </c>
     </row>
     <row r="40" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C40" s="21"/>
-      <c r="D40" s="16"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="19"/>
-      <c r="K40" s="18"/>
-      <c r="L40" s="18"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="16"/>
+      <c r="C40" s="20">
+        <v>45297</v>
+      </c>
+      <c r="D40" s="16">
+        <v>5.851</v>
+      </c>
+      <c r="E40">
+        <v>8.8020000000000008E-3</v>
+      </c>
+      <c r="F40">
+        <v>1710</v>
+      </c>
+      <c r="G40">
+        <v>8426</v>
+      </c>
+      <c r="H40">
+        <v>1.2643616490095195E-5</v>
+      </c>
+      <c r="I40" s="19">
+        <v>2.4750531543066637E-5</v>
+      </c>
+      <c r="J40" s="16">
+        <v>1.812754</v>
+      </c>
+      <c r="K40" s="16">
+        <v>6.402980390116519</v>
+      </c>
+      <c r="L40" s="16">
+        <v>2.7700364358100433</v>
+      </c>
+      <c r="M40" s="16">
+        <v>13.620893684280908</v>
+      </c>
+      <c r="N40" s="16">
+        <v>4.275317664330883</v>
+      </c>
     </row>
     <row r="41" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C41" s="21"/>
-      <c r="D41" s="16"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="19"/>
-      <c r="K41" s="18"/>
-      <c r="L41" s="18"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="16"/>
+      <c r="C41" s="20">
+        <v>45304</v>
+      </c>
+      <c r="D41" s="16">
+        <v>6.62</v>
+      </c>
+      <c r="E41">
+        <v>7.587E-3</v>
+      </c>
+      <c r="F41">
+        <v>1700</v>
+      </c>
+      <c r="G41">
+        <v>8419</v>
+      </c>
+      <c r="H41" s="19">
+        <v>1.265664078999726E-5</v>
+      </c>
+      <c r="I41" s="19">
+        <v>2.4759648552998081E-5</v>
+      </c>
+      <c r="J41" s="16">
+        <v>1.830829</v>
+      </c>
+      <c r="K41" s="16">
+        <v>7.1541841350661581</v>
+      </c>
+      <c r="L41" s="16">
+        <v>2.9404902626861738</v>
+      </c>
+      <c r="M41" s="16">
+        <v>12.202445646007522</v>
+      </c>
+      <c r="N41" s="16">
+        <v>3.9928078519637462</v>
+      </c>
     </row>
     <row r="42" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C42" s="21"/>
-      <c r="D42" s="16"/>
-      <c r="H42" s="19"/>
-      <c r="I42" s="19"/>
-      <c r="K42" s="18"/>
-      <c r="L42" s="18"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="16"/>
+      <c r="C42" s="20">
+        <v>45312</v>
+      </c>
+      <c r="D42" s="16">
+        <v>2.97</v>
+      </c>
+      <c r="E42">
+        <v>1.0026999999999999E-2</v>
+      </c>
+      <c r="F42">
+        <v>1678</v>
+      </c>
+      <c r="G42">
+        <v>8412</v>
+      </c>
+      <c r="H42" s="19">
+        <v>1.2669687036422975E-5</v>
+      </c>
+      <c r="I42" s="19">
+        <v>2.476878092549608E-5</v>
+      </c>
+      <c r="J42" s="16">
+        <v>1.844179</v>
+      </c>
+      <c r="K42" s="16">
+        <v>5.8706479383376529</v>
+      </c>
+      <c r="L42" s="16">
+        <v>2.6831138758352449</v>
+      </c>
+      <c r="M42" s="16">
+        <v>24.654472598325295</v>
+      </c>
+      <c r="N42" s="16">
+        <v>6.596817383838383</v>
+      </c>
     </row>
     <row r="43" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C43" s="21"/>
-      <c r="D43" s="16"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="19"/>
-      <c r="K43" s="18"/>
-      <c r="L43" s="18"/>
-      <c r="M43" s="16"/>
-      <c r="N43" s="16"/>
+      <c r="C43" s="20">
+        <v>45332</v>
+      </c>
+      <c r="D43" s="16">
+        <v>1.8424</v>
+      </c>
+      <c r="E43">
+        <v>8.9599999999999992E-3</v>
+      </c>
+      <c r="F43">
+        <v>1625</v>
+      </c>
+      <c r="G43">
+        <v>8394</v>
+      </c>
+      <c r="H43" s="19">
+        <v>1.2703335492640732E-5</v>
+      </c>
+      <c r="I43" s="19">
+        <v>2.4792334844848513E-5</v>
+      </c>
+      <c r="J43" s="16">
+        <v>1.877149</v>
+      </c>
+      <c r="K43" s="16">
+        <v>6.3788283922631779</v>
+      </c>
+      <c r="L43" s="16">
+        <v>2.8139793571428573</v>
+      </c>
+      <c r="M43" s="16">
+        <v>37.452730823356418</v>
+      </c>
+      <c r="N43" s="16">
+        <v>9.2806715792444638</v>
+      </c>
     </row>
     <row r="44" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C44" s="21"/>
-      <c r="D44" s="16"/>
-      <c r="H44" s="19"/>
-      <c r="I44" s="19"/>
-      <c r="K44" s="18"/>
-      <c r="L44" s="18"/>
-      <c r="M44" s="16"/>
-      <c r="N44" s="16"/>
+      <c r="C44" s="20">
+        <v>45360</v>
+      </c>
+      <c r="D44" s="16">
+        <v>2.3159999999999998</v>
+      </c>
+      <c r="E44">
+        <v>1.0128E-2</v>
+      </c>
+      <c r="F44">
+        <v>1582</v>
+      </c>
+      <c r="G44">
+        <v>8362</v>
+      </c>
+      <c r="I44" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J44" s="16">
+        <v>1.9220429999999999</v>
+      </c>
+      <c r="K44" s="16">
+        <v>8.1318654487565443</v>
+      </c>
+      <c r="L44" s="16">
+        <v>2.7476749115323855</v>
+      </c>
+      <c r="M44" s="16">
+        <v>44.88268865885663</v>
+      </c>
+      <c r="N44" s="16">
+        <v>7.6339100120898102</v>
+      </c>
     </row>
     <row r="45" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C45" s="21"/>
-      <c r="D45" s="16"/>
+      <c r="C45" s="20">
+        <v>45393</v>
+      </c>
+      <c r="D45" s="16">
+        <v>11.291</v>
+      </c>
+      <c r="E45">
+        <v>2.6429999999999999E-2</v>
+      </c>
+      <c r="F45">
+        <v>1705</v>
+      </c>
+      <c r="G45">
+        <v>8342</v>
+      </c>
       <c r="H45" s="19"/>
-      <c r="I45" s="19"/>
-      <c r="K45" s="18"/>
-      <c r="L45" s="18"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="16"/>
+      <c r="I45" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J45" s="16">
+        <v>1.9546349999999999</v>
+      </c>
+      <c r="K45" s="16">
+        <v>4.3342446012488196</v>
+      </c>
+      <c r="L45" s="16">
+        <v>2.2702611823685204</v>
+      </c>
+      <c r="M45" s="16">
+        <v>11.451818987469288</v>
+      </c>
+      <c r="N45" s="16">
+        <v>3.2143205902931538</v>
+      </c>
     </row>
     <row r="46" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C46" s="21"/>
-      <c r="D46" s="16"/>
-      <c r="H46" s="19"/>
-      <c r="I46" s="19"/>
-      <c r="K46" s="18"/>
-      <c r="L46" s="18"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="16"/>
+      <c r="C46" s="20">
+        <v>45423</v>
+      </c>
+      <c r="D46" s="16">
+        <v>3.21</v>
+      </c>
+      <c r="E46">
+        <v>1.2531E-2</v>
+      </c>
+      <c r="F46">
+        <v>1512</v>
+      </c>
+      <c r="G46">
+        <v>8294</v>
+      </c>
+      <c r="I46" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J46">
+        <v>2.0023599999999999</v>
+      </c>
+      <c r="K46" s="16">
+        <v>7.0213594223131661</v>
+      </c>
+      <c r="L46" s="16">
+        <v>2.66423854121778</v>
+      </c>
+      <c r="M46" s="16">
+        <v>31.626764866866512</v>
+      </c>
+      <c r="N46" s="16">
+        <v>5.9090665420560748</v>
+      </c>
     </row>
     <row r="47" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C47" s="21"/>
-      <c r="D47" s="16"/>
-      <c r="H47" s="19"/>
-      <c r="I47" s="19"/>
-      <c r="K47" s="18"/>
-      <c r="L47" s="18"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="16"/>
+      <c r="C47" s="20">
+        <v>45425</v>
+      </c>
+      <c r="D47" s="16">
+        <v>5.9749999999999996</v>
+      </c>
+      <c r="E47">
+        <v>1.0094000000000001E-2</v>
+      </c>
+      <c r="F47">
+        <v>1507</v>
+      </c>
+      <c r="G47">
+        <v>8285</v>
+      </c>
+      <c r="I47" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J47">
+        <v>2.0054349999999999</v>
+      </c>
+      <c r="K47" s="16">
+        <v>8.2361742273634118</v>
+      </c>
+      <c r="L47" s="16">
+        <v>2.8262196245294233</v>
+      </c>
+      <c r="M47" s="16">
+        <v>17.868175454198575</v>
+      </c>
+      <c r="N47" s="16">
+        <v>4.0950575941422596</v>
+      </c>
     </row>
     <row r="48" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C48" s="21"/>
-      <c r="D48" s="16"/>
-      <c r="H48" s="19"/>
-      <c r="I48" s="19"/>
-      <c r="K48" s="18"/>
-      <c r="L48" s="18"/>
-      <c r="M48" s="16"/>
-      <c r="N48" s="16"/>
+      <c r="C48" s="20">
+        <v>45446</v>
+      </c>
+      <c r="D48" s="16">
+        <v>2.1850000000000001</v>
+      </c>
+      <c r="E48">
+        <v>1.4767000000000001E-2</v>
+      </c>
+      <c r="F48">
+        <v>1445</v>
+      </c>
+      <c r="G48">
+        <v>8267</v>
+      </c>
+      <c r="I48" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J48">
+        <v>2.0328499999999998</v>
+      </c>
+      <c r="K48" s="16">
+        <v>6.2918790350786411</v>
+      </c>
+      <c r="L48" s="16">
+        <v>2.5926793492246221</v>
+      </c>
+      <c r="M48" s="16">
+        <v>43.625757617690667</v>
+      </c>
+      <c r="N48" s="16">
+        <v>7.5000422196796341</v>
+      </c>
     </row>
     <row r="49" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C49" s="21"/>
-      <c r="D49" s="16"/>
-      <c r="H49" s="19"/>
-      <c r="I49" s="19"/>
-      <c r="K49" s="18"/>
-      <c r="L49" s="18"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="16"/>
+      <c r="C49" s="20">
+        <v>45561</v>
+      </c>
+      <c r="D49" s="16">
+        <v>7.94</v>
+      </c>
+      <c r="E49">
+        <v>7.6049999999999998E-3</v>
+      </c>
+      <c r="F49">
+        <v>1305</v>
+      </c>
+      <c r="G49">
+        <v>8143</v>
+      </c>
+      <c r="I49" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J49">
+        <v>2.1853500000000001</v>
+      </c>
+      <c r="K49" s="16">
+        <v>10.455314728600433</v>
+      </c>
+      <c r="L49" s="16">
+        <v>3.2560929322813941</v>
+      </c>
+      <c r="M49" s="16">
+        <v>12.522311171047004</v>
+      </c>
+      <c r="N49" s="16">
+        <v>3.5237146095717886</v>
+      </c>
     </row>
     <row r="50" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C50" s="21"/>
-      <c r="D50" s="16"/>
-      <c r="H50" s="19"/>
-      <c r="I50" s="19"/>
-      <c r="K50" s="18"/>
-      <c r="L50" s="18"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="16"/>
+      <c r="C50" s="20">
+        <v>45565</v>
+      </c>
+      <c r="D50" s="16">
+        <v>4.0650000000000004</v>
+      </c>
+      <c r="E50">
+        <v>8.4709999999999994E-3</v>
+      </c>
+      <c r="F50">
+        <v>1301</v>
+      </c>
+      <c r="G50">
+        <v>8140</v>
+      </c>
+      <c r="I50" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J50">
+        <v>2.1905600000000001</v>
+      </c>
+      <c r="K50" s="16">
+        <v>9.6150767938857626</v>
+      </c>
+      <c r="L50" s="16">
+        <v>3.1514855105654584</v>
+      </c>
+      <c r="M50" s="16">
+        <v>22.319440534088361</v>
+      </c>
+      <c r="N50" s="16">
+        <v>4.7957604920049199</v>
+      </c>
     </row>
     <row r="51" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C51" s="21"/>
-      <c r="D51" s="16"/>
-      <c r="H51" s="19"/>
-      <c r="I51" s="19"/>
-      <c r="K51" s="18"/>
-      <c r="L51" s="18"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="16"/>
+      <c r="C51" s="20">
+        <v>45573</v>
+      </c>
+      <c r="D51" s="16">
+        <v>3.8</v>
+      </c>
+      <c r="E51">
+        <v>6.62E-3</v>
+      </c>
+      <c r="F51">
+        <v>1295</v>
+      </c>
+      <c r="G51">
+        <v>8138</v>
+      </c>
+      <c r="I51" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J51">
+        <v>2.2009400000000001</v>
+      </c>
+      <c r="K51" s="16">
+        <v>11.701405522810617</v>
+      </c>
+      <c r="L51" s="16">
+        <v>3.4302451359516617</v>
+      </c>
+      <c r="M51" s="16">
+        <v>23.634240231711352</v>
+      </c>
+      <c r="N51" s="16">
+        <v>4.9742847368421055</v>
+      </c>
     </row>
     <row r="52" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="H52" s="19"/>
-      <c r="I52" s="19"/>
-      <c r="K52" s="18"/>
-      <c r="L52" s="18"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="16"/>
+      <c r="C52" s="20">
+        <v>45578</v>
+      </c>
+      <c r="D52" s="16">
+        <v>3.3170000000000002</v>
+      </c>
+      <c r="E52">
+        <v>7.2560000000000003E-3</v>
+      </c>
+      <c r="F52">
+        <v>1292</v>
+      </c>
+      <c r="G52">
+        <v>8136</v>
+      </c>
+      <c r="I52" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J52">
+        <v>2.2074099999999999</v>
+      </c>
+      <c r="K52" s="16">
+        <v>10.875144531560956</v>
+      </c>
+      <c r="L52" s="16">
+        <v>3.3286889415656007</v>
+      </c>
+      <c r="M52" s="16">
+        <v>26.704805729641279</v>
+      </c>
+      <c r="N52" s="16">
+        <v>5.3764519053361468</v>
+      </c>
     </row>
     <row r="53" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C53" s="2"/>
-      <c r="E53" s="18"/>
-      <c r="H53" s="19"/>
-      <c r="I53" s="19"/>
-      <c r="K53" s="18"/>
-      <c r="L53" s="18"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="16"/>
+      <c r="C53" s="20">
+        <v>45720</v>
+      </c>
+      <c r="D53" s="16">
+        <v>1.9146000000000001</v>
+      </c>
+      <c r="E53">
+        <v>8.1200000000000005E-3</v>
+      </c>
+      <c r="F53">
+        <v>1158</v>
+      </c>
+      <c r="G53">
+        <v>8050</v>
+      </c>
+      <c r="I53" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J53">
+        <v>2.3809999999999998</v>
+      </c>
+      <c r="K53" s="16">
+        <v>10.126453418843138</v>
+      </c>
+      <c r="L53" s="16">
+        <v>3.3723793103448272</v>
+      </c>
+      <c r="M53" s="16">
+        <v>40.420375681210324</v>
+      </c>
+      <c r="N53" s="16">
+        <v>7.2498498903165149</v>
+      </c>
     </row>
     <row r="54" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C54" s="2"/>
-      <c r="D54" s="18"/>
-      <c r="E54" s="18"/>
-      <c r="H54" s="19"/>
-      <c r="I54" s="19"/>
-      <c r="K54" s="18"/>
-      <c r="L54" s="18"/>
-      <c r="M54" s="16"/>
-      <c r="N54" s="16"/>
+      <c r="C54" s="20">
+        <v>45809</v>
+      </c>
+      <c r="D54" s="16">
+        <v>0.87960000000000005</v>
+      </c>
+      <c r="E54">
+        <v>6.7609999999999996E-3</v>
+      </c>
+      <c r="F54">
+        <v>1145</v>
+      </c>
+      <c r="G54">
+        <v>7900</v>
+      </c>
+      <c r="I54" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J54">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="K54" s="16">
+        <v>11.772334234729522</v>
+      </c>
+      <c r="L54" s="16">
+        <v>3.6384662032243753</v>
+      </c>
+      <c r="M54" s="16">
+        <v>84.339689195489072</v>
+      </c>
+      <c r="N54" s="16">
+        <v>12.753651659845385</v>
+      </c>
+    </row>
+    <row r="55" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C55" s="20">
+        <v>45871</v>
+      </c>
+      <c r="D55" s="16">
+        <v>1.32</v>
+      </c>
+      <c r="E55">
+        <v>6.9880000000000003E-3</v>
+      </c>
+      <c r="F55">
+        <v>1120</v>
+      </c>
+      <c r="G55">
+        <v>7810</v>
+      </c>
+      <c r="I55" s="19">
+        <v>1.59E-5</v>
+      </c>
+      <c r="J55">
+        <v>2.5457049609016398</v>
+      </c>
+      <c r="K55" s="16">
+        <v>11.545859763564245</v>
+      </c>
+      <c r="L55" s="16">
+        <v>3.6633351841414794</v>
+      </c>
+      <c r="M55" s="16">
+        <v>55.909531909634246</v>
+      </c>
+      <c r="N55" s="16">
+        <v>9.1723716275683067</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix Date & Well name not visible
</commit_message>
<xml_diff>
--- a/data/S001.xlsx
+++ b/data/S001.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://odsi2005-my.sharepoint.com/personal/ibrahim_eltaleb_odsi-energy_com/Documents/ODSI_Desktop/Python/Stramlit/Dash_ODSI/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="8_{6132AEC3-1CAB-4FBA-A026-50CE20EF1FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86AA71A3-6283-4AD6-9803-63D9253B0DBE}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{6132AEC3-1CAB-4FBA-A026-50CE20EF1FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D80C1554-8A74-4EFD-9252-510DF9B5FE33}"/>
   <bookViews>
     <workbookView xWindow="2616" yWindow="2616" windowWidth="23040" windowHeight="13608" activeTab="2" xr2:uid="{92B28833-6805-4A4F-8867-695E222A4EA9}"/>
   </bookViews>
@@ -37277,7 +37277,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64D45957-36EC-4E57-B84E-45135FEB24AC}">
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:R55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -37285,7 +37285,7 @@
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="K1" t="s">
         <v>59</v>
       </c>
@@ -37293,7 +37293,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C2" s="15"/>
       <c r="J2" s="16"/>
       <c r="K2" t="s">
@@ -37309,7 +37309,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>63</v>
       </c>
@@ -37353,7 +37353,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>77</v>
       </c>
@@ -37397,7 +37397,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>84</v>
       </c>
@@ -37426,19 +37426,23 @@
         <v>3.8635999999999997E-2</v>
       </c>
       <c r="K5" s="16">
-        <v>2.0301248201269537</v>
+        <v>5.4399247245784723</v>
       </c>
       <c r="L5" s="16">
-        <v>0.63594322154222771</v>
+        <v>1.7719559212517029</v>
       </c>
       <c r="M5" s="16">
-        <v>2.0943556985273259</v>
+        <v>12.228941964492908</v>
       </c>
       <c r="N5" s="16">
-        <v>0.65520798824681681</v>
-      </c>
+        <v>3.4494658187873735</v>
+      </c>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="16"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -37467,19 +37471,23 @@
         <v>0.20100000000000001</v>
       </c>
       <c r="K6" s="16">
-        <v>4.0041275544137367</v>
+        <v>5.5159059002618864</v>
       </c>
       <c r="L6" s="16">
-        <v>1.2566760665220535</v>
+        <v>1.8239560175387686</v>
       </c>
       <c r="M6" s="16">
-        <v>5.3365828204904329</v>
+        <v>13.76757826256433</v>
       </c>
       <c r="N6" s="16">
-        <v>1.6265403726708076</v>
-      </c>
+        <v>3.8332765845460575</v>
+      </c>
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>86</v>
       </c>
@@ -37511,19 +37519,23 @@
         <v>0.29899999999999999</v>
       </c>
       <c r="K7" s="16">
-        <v>4.6009024507279497</v>
+        <v>5.4548123611099149</v>
       </c>
       <c r="L7" s="16">
-        <v>1.4491152604887043</v>
+        <v>1.8376622984239761</v>
       </c>
       <c r="M7" s="16">
-        <v>7.5106618479995468</v>
+        <v>15.041882292890739</v>
       </c>
       <c r="N7" s="16">
-        <v>2.2270405448210324</v>
-      </c>
+        <v>4.1399338056706645</v>
+      </c>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>88</v>
       </c>
@@ -37555,19 +37567,23 @@
         <v>0.377</v>
       </c>
       <c r="K8" s="16">
-        <v>4.4621380803155093</v>
+        <v>5.3491301684394994</v>
       </c>
       <c r="L8" s="16">
-        <v>1.4374449171319685</v>
+        <v>1.8385297200802457</v>
       </c>
       <c r="M8" s="16">
-        <v>9.2447120071420521</v>
+        <v>16.269464320058695</v>
       </c>
       <c r="N8" s="16">
-        <v>2.6789344608879491</v>
-      </c>
+        <v>4.4243117854018488</v>
+      </c>
+      <c r="O8" s="16"/>
+      <c r="P8" s="16"/>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>90</v>
       </c>
@@ -37599,19 +37615,23 @@
         <v>0.48899999999999999</v>
       </c>
       <c r="K9" s="16">
-        <v>4.9867925005573994</v>
+        <v>5.0692608975150222</v>
       </c>
       <c r="L9" s="16">
-        <v>1.6265974731023589</v>
+        <v>1.7958242391083155</v>
       </c>
       <c r="M9" s="16">
-        <v>10.463479944997566</v>
+        <v>17.469736224295804</v>
       </c>
       <c r="N9" s="16">
-        <v>3.0117804927713299</v>
-      </c>
+        <v>4.6926782003936403</v>
+      </c>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="16"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>92</v>
       </c>
@@ -37643,19 +37663,23 @@
         <v>0.55800000000000005</v>
       </c>
       <c r="K10" s="16">
-        <v>5.4469665324725387</v>
+        <v>4.7809715975103542</v>
       </c>
       <c r="L10" s="16">
-        <v>1.7802222222222224</v>
+        <v>1.7505648950690567</v>
       </c>
       <c r="M10" s="16">
-        <v>12.932360213695913</v>
+        <v>18.467046193952918</v>
       </c>
       <c r="N10" s="16">
-        <v>3.6515409229141875</v>
-      </c>
+        <v>4.9106228322762062</v>
+      </c>
+      <c r="O10" s="16"/>
+      <c r="P10" s="16"/>
+      <c r="Q10" s="16"/>
+      <c r="R10" s="16"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>94</v>
       </c>
@@ -37684,19 +37708,23 @@
         <v>0.61599999999999999</v>
       </c>
       <c r="K11" s="16">
-        <v>5.6618488513973206</v>
+        <v>4.5008952998919414</v>
       </c>
       <c r="L11" s="16">
-        <v>1.8632853464681518</v>
+        <v>1.7098399060731391</v>
       </c>
       <c r="M11" s="16">
-        <v>12.324986022970865</v>
+        <v>19.101391551023013</v>
       </c>
       <c r="N11" s="16">
-        <v>3.5103488238668965</v>
-      </c>
+        <v>5.045968933984315</v>
+      </c>
+      <c r="O11" s="16"/>
+      <c r="P11" s="16"/>
+      <c r="Q11" s="16"/>
+      <c r="R11" s="16"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>95</v>
       </c>
@@ -37725,19 +37753,23 @@
         <v>0.63</v>
       </c>
       <c r="K12" s="16">
-        <v>9.1024219000692526</v>
+        <v>4.2138267435969858</v>
       </c>
       <c r="L12" s="16">
-        <v>2.7217810795561408</v>
+        <v>1.6707638732644521</v>
       </c>
       <c r="M12" s="16">
-        <v>13.941163861329127</v>
+        <v>20.340614320910049</v>
       </c>
       <c r="N12" s="16">
-        <v>3.9164322669970124</v>
-      </c>
+        <v>5.3145078848961456</v>
+      </c>
+      <c r="O12" s="16"/>
+      <c r="P12" s="16"/>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="16"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -37766,19 +37798,23 @@
         <v>0.67800000000000005</v>
       </c>
       <c r="K13" s="16">
-        <v>5.7843289549548373</v>
+        <v>3.9775845489109489</v>
       </c>
       <c r="L13" s="16">
-        <v>1.927886156648452</v>
+        <v>1.6480634885625798</v>
       </c>
       <c r="M13" s="16">
-        <v>16.048830830140322</v>
+        <v>21.959969854562793</v>
       </c>
       <c r="N13" s="16">
-        <v>4.4403484190410012</v>
-      </c>
+        <v>5.6685219546079102</v>
+      </c>
+      <c r="O13" s="16"/>
+      <c r="P13" s="16"/>
+      <c r="Q13" s="16"/>
+      <c r="R13" s="16"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>87</v>
       </c>
@@ -37807,19 +37843,23 @@
         <v>0.72845860920204608</v>
       </c>
       <c r="K14" s="16">
-        <v>4.1099984829781517</v>
+        <v>3.8810368663425159</v>
       </c>
       <c r="L14" s="16">
-        <v>1.5513697623211387</v>
+        <v>1.663798361303392</v>
       </c>
       <c r="M14" s="16">
-        <v>16.468385635968495</v>
+        <v>23.204114950461953</v>
       </c>
       <c r="N14" s="16">
-        <v>4.5588323392455878</v>
-      </c>
+        <v>5.9465476687765211</v>
+      </c>
+      <c r="O14" s="16"/>
+      <c r="P14" s="16"/>
+      <c r="Q14" s="16"/>
+      <c r="R14" s="16"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>97</v>
       </c>
@@ -37848,19 +37888,23 @@
         <v>0.81045860920204604</v>
       </c>
       <c r="K15" s="16">
-        <v>5.4860861675183381</v>
+        <v>3.8889223986160086</v>
       </c>
       <c r="L15" s="16">
-        <v>1.9324303808472956</v>
+        <v>1.7072123889701349</v>
       </c>
       <c r="M15" s="16">
-        <v>16.40016838182482</v>
+        <v>24.442407912098947</v>
       </c>
       <c r="N15" s="16">
-        <v>4.5513926495778945</v>
-      </c>
+        <v>6.2318467393229158</v>
+      </c>
+      <c r="O15" s="16"/>
+      <c r="P15" s="16"/>
+      <c r="Q15" s="16"/>
+      <c r="R15" s="16"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>98</v>
       </c>
@@ -37889,19 +37933,23 @@
         <v>0.84445860920204607</v>
       </c>
       <c r="K16" s="16">
-        <v>3.4777168544655259</v>
+        <v>4.0876064899624192</v>
       </c>
       <c r="L16" s="16">
-        <v>1.441870763491615</v>
+        <v>1.7936626723055722</v>
       </c>
       <c r="M16" s="16">
-        <v>22.168556460557404</v>
+        <v>27.69008975473087</v>
       </c>
       <c r="N16" s="16">
-        <v>5.6822960140879086</v>
-      </c>
+        <v>6.9522981836056594</v>
+      </c>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>89</v>
       </c>
@@ -37930,19 +37978,23 @@
         <v>0.86845860920204609</v>
       </c>
       <c r="K17" s="16">
-        <v>4.2652019735612567</v>
+        <v>4.39750182071342</v>
       </c>
       <c r="L17" s="16">
-        <v>1.632223726961435</v>
+        <v>1.9062435931539963</v>
       </c>
       <c r="M17" s="16">
-        <v>25.109302933522905</v>
+        <v>31.263294300695769</v>
       </c>
       <c r="N17" s="16">
-        <v>6.3190650677928986</v>
-      </c>
+        <v>7.7428685430076811</v>
+      </c>
+      <c r="O17" s="16"/>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="16"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C18" s="20">
         <v>44915</v>
       </c>
@@ -37968,19 +38020,23 @@
         <v>0.91500000000000004</v>
       </c>
       <c r="K18" s="16">
-        <v>3.718182073885004</v>
+        <v>4.7104745634996545</v>
       </c>
       <c r="L18" s="16">
-        <v>1.5404125412541254</v>
+        <v>2.0188221889874063</v>
       </c>
       <c r="M18" s="16">
-        <v>16.313544635508155</v>
+        <v>34.950051997072364</v>
       </c>
       <c r="N18" s="16">
-        <v>4.3505395683453241</v>
-      </c>
+        <v>8.5549853238982578</v>
+      </c>
+      <c r="O18" s="16"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C19" s="20">
         <v>44932</v>
       </c>
@@ -38006,19 +38062,23 @@
         <v>0.97699999999999998</v>
       </c>
       <c r="K19" s="16">
-        <v>3.9841736392239597</v>
+        <v>5.0511561362856501</v>
       </c>
       <c r="L19" s="16">
-        <v>1.6444246731097214</v>
+        <v>2.1348139660410452</v>
       </c>
       <c r="M19" s="16">
-        <v>21.587908712110895</v>
+        <v>38.733254115700703</v>
       </c>
       <c r="N19" s="16">
-        <v>5.5514711347047117</v>
-      </c>
+        <v>9.3876321818038981</v>
+      </c>
+      <c r="O19" s="16"/>
+      <c r="P19" s="16"/>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="16"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C20" s="20">
         <v>44944</v>
       </c>
@@ -38044,19 +38104,23 @@
         <v>1.02</v>
       </c>
       <c r="K20" s="16">
-        <v>3.0201224866971721</v>
+        <v>5.338423994794268</v>
       </c>
       <c r="L20" s="16">
-        <v>1.4621800947867298</v>
+        <v>2.2348954668672016</v>
       </c>
       <c r="M20" s="16">
-        <v>21.738265477920507</v>
+        <v>41.644768869925542</v>
       </c>
       <c r="N20" s="16">
-        <v>5.6003217821782183</v>
-      </c>
+        <v>10.026969296032034</v>
+      </c>
+      <c r="O20" s="16"/>
+      <c r="P20" s="16"/>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="16"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C21" s="20">
         <v>44965</v>
       </c>
@@ -38082,19 +38146,23 @@
         <v>1.0900000000000001</v>
       </c>
       <c r="K21" s="16">
-        <v>4.4631065658972542</v>
+        <v>5.4512812807605684</v>
       </c>
       <c r="L21" s="16">
-        <v>1.8301574803149607</v>
+        <v>2.293610598296262</v>
       </c>
       <c r="M21" s="16">
-        <v>20.854197900355942</v>
+        <v>42.302217616898837</v>
       </c>
       <c r="N21" s="16">
-        <v>5.4268386478719028</v>
-      </c>
+        <v>10.178078086938125</v>
+      </c>
+      <c r="O21" s="16"/>
+      <c r="P21" s="16"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="16"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C22" s="20">
         <v>45003</v>
       </c>
@@ -38120,19 +38188,23 @@
         <v>1.182714</v>
       </c>
       <c r="K22" s="16">
-        <v>3.7169280514322001</v>
+        <v>5.5438570469012403</v>
       </c>
       <c r="L22" s="16">
-        <v>1.7383702179138734</v>
+        <v>2.3437604805704773</v>
       </c>
       <c r="M22" s="16">
-        <v>16.595624121013064</v>
+        <v>42.18956014361116</v>
       </c>
       <c r="N22" s="16">
-        <v>4.5621757072888993</v>
-      </c>
+        <v>10.162059113929953</v>
+      </c>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16"/>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="16"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C23" s="20">
         <v>45039</v>
       </c>
@@ -38158,19 +38230,23 @@
         <v>1.28</v>
       </c>
       <c r="K23" s="16">
-        <v>3.4776113618691351</v>
+        <v>5.5926757200236228</v>
       </c>
       <c r="L23" s="16">
-        <v>1.758578947368421</v>
+        <v>2.3802745716689988</v>
       </c>
       <c r="M23" s="16">
-        <v>43.976449316314621</v>
+        <v>41.340856871470351</v>
       </c>
       <c r="N23" s="16">
-        <v>10.578105263157894</v>
-      </c>
+        <v>9.9882622127543517</v>
+      </c>
+      <c r="O23" s="16"/>
+      <c r="P23" s="16"/>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C24" s="20">
         <v>45059</v>
       </c>
@@ -38196,19 +38272,23 @@
         <v>1.3380000000000001</v>
       </c>
       <c r="K24" s="16">
-        <v>3.833096106648838</v>
+        <v>5.4926469210730158</v>
       </c>
       <c r="L24" s="16">
-        <v>1.8780360144057624</v>
+        <v>2.3816358341194457</v>
       </c>
       <c r="M24" s="16">
-        <v>46.636789700325899</v>
+        <v>38.255295059448208</v>
       </c>
       <c r="N24" s="16">
-        <v>11.142423076923077</v>
-      </c>
+        <v>9.3354863410009656</v>
+      </c>
+      <c r="O24" s="16"/>
+      <c r="P24" s="16"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C25" s="20">
         <v>45085</v>
       </c>
@@ -38234,19 +38314,23 @@
         <v>1.397</v>
       </c>
       <c r="K25" s="16">
-        <v>3.7706830448933779</v>
+        <v>5.3882426215467571</v>
       </c>
       <c r="L25" s="16">
-        <v>1.9100330398993941</v>
+        <v>2.3802332123593519</v>
       </c>
       <c r="M25" s="16">
-        <v>17.897987039970889</v>
+        <v>35.279168314456598</v>
       </c>
       <c r="N25" s="16">
-        <v>4.9634203612479473</v>
-      </c>
+        <v>8.7066132828196583</v>
+      </c>
+      <c r="O25" s="16"/>
+      <c r="P25" s="16"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C26" s="15">
         <v>45104</v>
       </c>
@@ -38272,19 +38356,23 @@
         <v>1.4470000000000001</v>
       </c>
       <c r="K26" s="16">
-        <v>6.5742882785044205</v>
+        <v>5.3072321300391199</v>
       </c>
       <c r="L26" s="16">
-        <v>2.5498500619578683</v>
+        <v>2.3822779464122021</v>
       </c>
       <c r="M26" s="16">
-        <v>20.88482633523704</v>
+        <v>31.72161292297039</v>
       </c>
       <c r="N26" s="16">
-        <v>5.6279640522875818</v>
-      </c>
+        <v>7.960207175899348</v>
+      </c>
+      <c r="O26" s="16"/>
+      <c r="P26" s="16"/>
+      <c r="Q26" s="16"/>
+      <c r="R26" s="16"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C27" s="15">
         <v>45114</v>
       </c>
@@ -38310,19 +38398,23 @@
         <v>1.4697</v>
       </c>
       <c r="K27" s="16">
-        <v>11.223045570594754</v>
+        <v>5.2453754357665634</v>
       </c>
       <c r="L27" s="16">
-        <v>3.552875355450237</v>
+        <v>2.3869543843485244</v>
       </c>
       <c r="M27" s="16">
-        <v>102.09070243695257</v>
+        <v>28.609058683361599</v>
       </c>
       <c r="N27" s="16">
-        <v>22.960909452201932</v>
-      </c>
+        <v>7.3058016672267545</v>
+      </c>
+      <c r="O27" s="16"/>
+      <c r="P27" s="16"/>
+      <c r="Q27" s="16"/>
+      <c r="R27" s="16"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C28" s="15">
         <v>45122</v>
       </c>
@@ -38348,19 +38440,23 @@
         <v>1.4887999999999999</v>
       </c>
       <c r="K28" s="16">
-        <v>5.4600972572315563</v>
+        <v>5.2718568122134473</v>
       </c>
       <c r="L28" s="16">
-        <v>2.3335541618273323</v>
+        <v>2.4098520659961187</v>
       </c>
       <c r="M28" s="16">
-        <v>62.335454545729569</v>
+        <v>26.36639253827056</v>
       </c>
       <c r="N28" s="16">
-        <v>14.43179100052938</v>
-      </c>
+        <v>6.8317168421215735</v>
+      </c>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C29" s="15">
         <v>45151</v>
       </c>
@@ -38386,19 +38482,23 @@
         <v>1.5504</v>
       </c>
       <c r="K29" s="16">
-        <v>4.9415822994899052</v>
+        <v>5.4895256852949945</v>
       </c>
       <c r="L29" s="16">
-        <v>2.2662297306285333</v>
+        <v>2.4734992751217995</v>
       </c>
       <c r="M29" s="16">
-        <v>49.864557156592014</v>
+        <v>25.860522171877278</v>
       </c>
       <c r="N29" s="16">
-        <v>11.748822570249336</v>
-      </c>
+        <v>6.7312867583125513</v>
+      </c>
+      <c r="O29" s="16"/>
+      <c r="P29" s="16"/>
+      <c r="Q29" s="16"/>
+      <c r="R29" s="16"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C30" s="15">
         <v>45162</v>
       </c>
@@ -38424,19 +38524,23 @@
         <v>1.5723</v>
       </c>
       <c r="K30" s="16">
-        <v>4.3307623227547865</v>
+        <v>5.7374507959306751</v>
       </c>
       <c r="L30" s="16">
-        <v>2.1527067796610169</v>
+        <v>2.5431270347164094</v>
       </c>
       <c r="M30" s="16">
-        <v>13.242085117530809</v>
+        <v>25.615410019080404</v>
       </c>
       <c r="N30" s="16">
-        <v>4.0277340813464235</v>
-      </c>
+        <v>6.6904037132337733</v>
+      </c>
+      <c r="O30" s="16"/>
+      <c r="P30" s="16"/>
+      <c r="Q30" s="16"/>
+      <c r="R30" s="16"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C31" s="20">
         <v>45168</v>
       </c>
@@ -38462,19 +38566,23 @@
         <v>1.5825</v>
       </c>
       <c r="K31" s="16">
-        <v>4.1971689953934135</v>
+        <v>5.969625063980085</v>
       </c>
       <c r="L31" s="16">
-        <v>2.1316054189728408</v>
+        <v>2.6090281211014483</v>
       </c>
       <c r="M31" s="16">
-        <v>13.680236439903693</v>
+        <v>26.298250650933078</v>
       </c>
       <c r="N31" s="16">
-        <v>4.1231399999999994</v>
-      </c>
+        <v>6.8439957456753797</v>
+      </c>
+      <c r="O31" s="16"/>
+      <c r="P31" s="16"/>
+      <c r="Q31" s="16"/>
+      <c r="R31" s="16"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="C32" s="20">
         <v>45181</v>
       </c>
@@ -38500,19 +38608,23 @@
         <v>1.6111899999999999</v>
       </c>
       <c r="K32" s="16">
-        <v>4.0955451363269697</v>
+        <v>6.1543238711883177</v>
       </c>
       <c r="L32" s="16">
-        <v>2.1318319208624281</v>
+        <v>2.665400415728556</v>
       </c>
       <c r="M32" s="16">
-        <v>36.976943135105891</v>
+        <v>26.996014349102545</v>
       </c>
       <c r="N32" s="16">
-        <v>9.0227284615384615</v>
-      </c>
+        <v>7.002262277727163</v>
+      </c>
+      <c r="O32" s="16"/>
+      <c r="P32" s="16"/>
+      <c r="Q32" s="16"/>
+      <c r="R32" s="16"/>
     </row>
-    <row r="33" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C33" s="20">
         <v>45204</v>
       </c>
@@ -38538,19 +38650,23 @@
         <v>1.65398</v>
       </c>
       <c r="K33" s="16">
-        <v>5.399397022402634</v>
+        <v>6.3356605718812542</v>
       </c>
       <c r="L33" s="16">
-        <v>2.4387971407462135</v>
+        <v>2.7100766927253024</v>
       </c>
       <c r="M33" s="16">
-        <v>27.690927297341009</v>
+        <v>27.046327877909423</v>
       </c>
       <c r="N33" s="16">
-        <v>7.1097790230286106</v>
-      </c>
+        <v>6.9474607496154031</v>
+      </c>
+      <c r="O33" s="16"/>
+      <c r="P33" s="16"/>
+      <c r="Q33" s="16"/>
+      <c r="R33" s="16"/>
     </row>
-    <row r="34" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C34" s="20">
         <v>45215</v>
       </c>
@@ -38576,19 +38692,23 @@
         <v>1.67466</v>
       </c>
       <c r="K34" s="16">
-        <v>5.3024802913654447</v>
+        <v>6.4141729150128501</v>
       </c>
       <c r="L34" s="16">
-        <v>2.4404906652436855</v>
+        <v>2.7291063896674976</v>
       </c>
       <c r="M34" s="16">
-        <v>20.453353637347583</v>
+        <v>27.543148999383966</v>
       </c>
       <c r="N34" s="16">
-        <v>5.6388308479678875</v>
-      </c>
+        <v>6.9685073560585495</v>
+      </c>
+      <c r="O34" s="16"/>
+      <c r="P34" s="16"/>
+      <c r="Q34" s="16"/>
+      <c r="R34" s="16"/>
     </row>
-    <row r="35" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C35" s="20">
         <v>45221</v>
       </c>
@@ -38614,19 +38734,23 @@
         <v>1.6836599999999999</v>
       </c>
       <c r="K35" s="16">
-        <v>5.8829809589978028</v>
+        <v>6.4562088611440052</v>
       </c>
       <c r="L35" s="16">
-        <v>2.5610987712743878</v>
+        <v>2.7325312461954705</v>
       </c>
       <c r="M35" s="16">
-        <v>9.2628218382173717</v>
+        <v>28.196974497563559</v>
       </c>
       <c r="N35" s="16">
-        <v>3.2673090031479539</v>
-      </c>
+        <v>6.9688519885038227</v>
+      </c>
+      <c r="O35" s="16"/>
+      <c r="P35" s="16"/>
+      <c r="Q35" s="16"/>
+      <c r="R35" s="16"/>
     </row>
-    <row r="36" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C36" s="20">
         <v>45229</v>
       </c>
@@ -38652,19 +38776,23 @@
         <v>1.6988300000000001</v>
       </c>
       <c r="K36" s="16">
-        <v>6.0046348677297354</v>
+        <v>6.5284728758591388</v>
       </c>
       <c r="L36" s="16">
-        <v>2.5960252650101312</v>
+        <v>2.7317686188041512</v>
       </c>
       <c r="M36" s="16">
-        <v>36.416644350539698</v>
+        <v>27.99136922000557</v>
       </c>
       <c r="N36" s="16">
-        <v>8.9329382802547777</v>
-      </c>
+        <v>6.7639525439464707</v>
+      </c>
+      <c r="O36" s="16"/>
+      <c r="P36" s="16"/>
+      <c r="Q36" s="16"/>
+      <c r="R36" s="16"/>
     </row>
-    <row r="37" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C37" s="20">
         <v>45248</v>
       </c>
@@ -38690,19 +38818,23 @@
         <v>1.7322310000000001</v>
       </c>
       <c r="K37" s="16">
-        <v>6.1397836499128946</v>
+        <v>6.5855631708666911</v>
       </c>
       <c r="L37" s="16">
-        <v>2.6579198696029507</v>
+        <v>2.7202500496014848</v>
       </c>
       <c r="M37" s="16">
-        <v>16.9475647315878</v>
+        <v>27.831137816154346</v>
       </c>
       <c r="N37" s="16">
-        <v>4.9278060053044772</v>
-      </c>
+        <v>6.4893371488704252</v>
+      </c>
+      <c r="O37" s="16"/>
+      <c r="P37" s="16"/>
+      <c r="Q37" s="16"/>
+      <c r="R37" s="16"/>
     </row>
-    <row r="38" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C38" s="20">
         <v>45263</v>
       </c>
@@ -38728,19 +38860,23 @@
         <v>1.75732</v>
       </c>
       <c r="K38" s="16">
-        <v>6.7256281896672938</v>
+        <v>6.6720009661869293</v>
       </c>
       <c r="L38" s="16">
-        <v>2.7867390358467246</v>
+        <v>2.7128303059756425</v>
       </c>
       <c r="M38" s="16">
-        <v>40.835071449998068</v>
+        <v>27.467251942721187</v>
       </c>
       <c r="N38" s="16">
-        <v>9.854116673035854</v>
-      </c>
+        <v>6.2354701294387045</v>
+      </c>
+      <c r="O38" s="16"/>
+      <c r="P38" s="16"/>
+      <c r="Q38" s="16"/>
+      <c r="R38" s="16"/>
     </row>
-    <row r="39" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C39" s="20">
         <v>45279</v>
       </c>
@@ -38766,19 +38902,23 @@
         <v>1.7849999999999999</v>
       </c>
       <c r="K39" s="16">
-        <v>6.4588838370320536</v>
+        <v>6.8971879591124736</v>
       </c>
       <c r="L39" s="16">
-        <v>2.7510957707095418</v>
+        <v>2.7268113203989159</v>
       </c>
       <c r="M39" s="16">
-        <v>48.044287522724105</v>
+        <v>27.182383911285065</v>
       </c>
       <c r="N39" s="16">
-        <v>11.346834138376762</v>
-      </c>
+        <v>5.9794138230864311</v>
+      </c>
+      <c r="O39" s="16"/>
+      <c r="P39" s="16"/>
+      <c r="Q39" s="16"/>
+      <c r="R39" s="16"/>
     </row>
-    <row r="40" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C40" s="20">
         <v>45297</v>
       </c>
@@ -38804,19 +38944,23 @@
         <v>1.812754</v>
       </c>
       <c r="K40" s="16">
-        <v>6.402980390116519</v>
+        <v>7.2480460994855562</v>
       </c>
       <c r="L40" s="16">
-        <v>2.7700364358100433</v>
+        <v>2.7592614916581337</v>
       </c>
       <c r="M40" s="16">
-        <v>13.620893684280908</v>
+        <v>26.78226127963611</v>
       </c>
       <c r="N40" s="16">
-        <v>4.275317664330883</v>
-      </c>
+        <v>5.7143240989485928</v>
+      </c>
+      <c r="O40" s="16"/>
+      <c r="P40" s="16"/>
+      <c r="Q40" s="16"/>
+      <c r="R40" s="16"/>
     </row>
-    <row r="41" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C41" s="20">
         <v>45304</v>
       </c>
@@ -38842,19 +38986,23 @@
         <v>1.830829</v>
       </c>
       <c r="K41" s="16">
-        <v>7.1541841350661581</v>
+        <v>7.6230539571704643</v>
       </c>
       <c r="L41" s="16">
-        <v>2.9404902626861738</v>
+        <v>2.8043589173226846</v>
       </c>
       <c r="M41" s="16">
-        <v>12.202445646007522</v>
+        <v>26.682094376469909</v>
       </c>
       <c r="N41" s="16">
-        <v>3.9928078519637462</v>
-      </c>
+        <v>5.5740923357477765</v>
+      </c>
+      <c r="O41" s="16"/>
+      <c r="P41" s="16"/>
+      <c r="Q41" s="16"/>
+      <c r="R41" s="16"/>
     </row>
-    <row r="42" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C42" s="20">
         <v>45312</v>
       </c>
@@ -38880,19 +39028,23 @@
         <v>1.844179</v>
       </c>
       <c r="K42" s="16">
-        <v>5.8706479383376529</v>
+        <v>8.1456445691711785</v>
       </c>
       <c r="L42" s="16">
-        <v>2.6831138758352449</v>
+        <v>2.8814432233512788</v>
       </c>
       <c r="M42" s="16">
-        <v>24.654472598325295</v>
+        <v>26.556019792311986</v>
       </c>
       <c r="N42" s="16">
-        <v>6.596817383838383</v>
-      </c>
+        <v>5.4541306911638241</v>
+      </c>
+      <c r="O42" s="16"/>
+      <c r="P42" s="16"/>
+      <c r="Q42" s="16"/>
+      <c r="R42" s="16"/>
     </row>
-    <row r="43" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C43" s="20">
         <v>45332</v>
       </c>
@@ -38918,19 +39070,23 @@
         <v>1.877149</v>
       </c>
       <c r="K43" s="16">
-        <v>6.3788283922631779</v>
+        <v>8.7044812866439436</v>
       </c>
       <c r="L43" s="16">
-        <v>2.8139793571428573</v>
+        <v>2.9749931541901571</v>
       </c>
       <c r="M43" s="16">
-        <v>37.452730823356418</v>
+        <v>27.739771678243635</v>
       </c>
       <c r="N43" s="16">
-        <v>9.2806715792444638</v>
-      </c>
+        <v>5.5170110055844033</v>
+      </c>
+      <c r="O43" s="16"/>
+      <c r="P43" s="16"/>
+      <c r="Q43" s="16"/>
+      <c r="R43" s="16"/>
     </row>
-    <row r="44" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C44" s="20">
         <v>45360</v>
       </c>
@@ -38953,19 +39109,23 @@
         <v>1.9220429999999999</v>
       </c>
       <c r="K44" s="16">
-        <v>8.1318654487565443</v>
+        <v>9.2524494211330275</v>
       </c>
       <c r="L44" s="16">
-        <v>2.7476749115323855</v>
+        <v>3.0777616831510817</v>
       </c>
       <c r="M44" s="16">
-        <v>44.88268865885663</v>
+        <v>29.932933277167113</v>
       </c>
       <c r="N44" s="16">
-        <v>7.6339100120898102</v>
-      </c>
+        <v>5.7518505931364707</v>
+      </c>
+      <c r="O44" s="16"/>
+      <c r="P44" s="16"/>
+      <c r="Q44" s="16"/>
+      <c r="R44" s="16"/>
     </row>
-    <row r="45" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C45" s="20">
         <v>45393</v>
       </c>
@@ -38989,19 +39149,23 @@
         <v>1.9546349999999999</v>
       </c>
       <c r="K45" s="16">
-        <v>4.3342446012488196</v>
+        <v>9.7870548511608195</v>
       </c>
       <c r="L45" s="16">
-        <v>2.2702611823685204</v>
+        <v>3.187824519156647</v>
       </c>
       <c r="M45" s="16">
-        <v>11.451818987469288</v>
+        <v>32.677003216164287</v>
       </c>
       <c r="N45" s="16">
-        <v>3.2143205902931538</v>
-      </c>
+        <v>6.1228008280257704</v>
+      </c>
+      <c r="O45" s="16"/>
+      <c r="P45" s="16"/>
+      <c r="Q45" s="16"/>
+      <c r="R45" s="16"/>
     </row>
-    <row r="46" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C46" s="20">
         <v>45423</v>
       </c>
@@ -39024,19 +39188,23 @@
         <v>2.0023599999999999</v>
       </c>
       <c r="K46" s="16">
-        <v>7.0213594223131661</v>
+        <v>10.272107526509748</v>
       </c>
       <c r="L46" s="16">
-        <v>2.66423854121778</v>
+        <v>3.2923447574873821</v>
       </c>
       <c r="M46" s="16">
-        <v>31.626764866866512</v>
+        <v>37.277532379829715</v>
       </c>
       <c r="N46" s="16">
-        <v>5.9090665420560748</v>
-      </c>
+        <v>6.7324071715376235</v>
+      </c>
+      <c r="O46" s="16"/>
+      <c r="P46" s="16"/>
+      <c r="Q46" s="16"/>
+      <c r="R46" s="16"/>
     </row>
-    <row r="47" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C47" s="20">
         <v>45425</v>
       </c>
@@ -39059,19 +39227,23 @@
         <v>2.0054349999999999</v>
       </c>
       <c r="K47" s="16">
-        <v>8.2361742273634118</v>
+        <v>10.688999546222073</v>
       </c>
       <c r="L47" s="16">
-        <v>2.8262196245294233</v>
+        <v>3.386439445252281</v>
       </c>
       <c r="M47" s="16">
-        <v>17.868175454198575</v>
+        <v>42.844047457802645</v>
       </c>
       <c r="N47" s="16">
-        <v>4.0950575941422596</v>
-      </c>
+        <v>7.4571925905646133</v>
+      </c>
+      <c r="O47" s="16"/>
+      <c r="P47" s="16"/>
+      <c r="Q47" s="16"/>
+      <c r="R47" s="16"/>
     </row>
-    <row r="48" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C48" s="20">
         <v>45446</v>
       </c>
@@ -39094,19 +39266,23 @@
         <v>2.0328499999999998</v>
       </c>
       <c r="K48" s="16">
-        <v>6.2918790350786411</v>
+        <v>10.974735758974131</v>
       </c>
       <c r="L48" s="16">
-        <v>2.5926793492246221</v>
+        <v>3.4629382794561523</v>
       </c>
       <c r="M48" s="16">
-        <v>43.625757617690667</v>
+        <v>46.833490821288535</v>
       </c>
       <c r="N48" s="16">
-        <v>7.5000422196796341</v>
-      </c>
+        <v>7.9815175527046343</v>
+      </c>
+      <c r="O48" s="16"/>
+      <c r="P48" s="16"/>
+      <c r="Q48" s="16"/>
+      <c r="R48" s="16"/>
     </row>
-    <row r="49" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C49" s="20">
         <v>45561</v>
       </c>
@@ -39129,19 +39305,23 @@
         <v>2.1853500000000001</v>
       </c>
       <c r="K49" s="16">
-        <v>10.455314728600433</v>
+        <v>11.144303135629396</v>
       </c>
       <c r="L49" s="16">
-        <v>3.2560929322813941</v>
+        <v>3.5073811231044956</v>
       </c>
       <c r="M49" s="16">
-        <v>12.522311171047004</v>
+        <v>49.843802216210364</v>
       </c>
       <c r="N49" s="16">
-        <v>3.5237146095717886</v>
-      </c>
+        <v>8.3740128041357345</v>
+      </c>
+      <c r="O49" s="16"/>
+      <c r="P49" s="16"/>
+      <c r="Q49" s="16"/>
+      <c r="R49" s="16"/>
     </row>
-    <row r="50" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C50" s="20">
         <v>45565</v>
       </c>
@@ -39164,19 +39344,23 @@
         <v>2.1905600000000001</v>
       </c>
       <c r="K50" s="16">
-        <v>9.6150767938857626</v>
+        <v>11.242573825044266</v>
       </c>
       <c r="L50" s="16">
-        <v>3.1514855105654584</v>
+        <v>3.5406482492649469</v>
       </c>
       <c r="M50" s="16">
-        <v>22.319440534088361</v>
+        <v>53.964396807322146</v>
       </c>
       <c r="N50" s="16">
-        <v>4.7957604920049199</v>
-      </c>
+        <v>8.9056795503559751</v>
+      </c>
+      <c r="O50" s="16"/>
+      <c r="P50" s="16"/>
+      <c r="Q50" s="16"/>
+      <c r="R50" s="16"/>
     </row>
-    <row r="51" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C51" s="20">
         <v>45573</v>
       </c>
@@ -39199,19 +39383,23 @@
         <v>2.2009400000000001</v>
       </c>
       <c r="K51" s="16">
-        <v>11.701405522810617</v>
+        <v>11.327472009979918</v>
       </c>
       <c r="L51" s="16">
-        <v>3.4302451359516617</v>
+        <v>3.5719272950518586</v>
       </c>
       <c r="M51" s="16">
-        <v>23.634240231711352</v>
+        <v>56.860534113900961</v>
       </c>
       <c r="N51" s="16">
-        <v>4.9742847368421055</v>
-      </c>
+        <v>9.2808155130533656</v>
+      </c>
+      <c r="O51" s="16"/>
+      <c r="P51" s="16"/>
+      <c r="Q51" s="16"/>
+      <c r="R51" s="16"/>
     </row>
-    <row r="52" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C52" s="20">
         <v>45578</v>
       </c>
@@ -39234,19 +39422,23 @@
         <v>2.2074099999999999</v>
       </c>
       <c r="K52" s="16">
-        <v>10.875144531560956</v>
+        <v>11.358280138899474</v>
       </c>
       <c r="L52" s="16">
-        <v>3.3286889415656007</v>
+        <v>3.5932533800534263</v>
       </c>
       <c r="M52" s="16">
-        <v>26.704805729641279</v>
+        <v>59.525235504991876</v>
       </c>
       <c r="N52" s="16">
-        <v>5.3764519053361468</v>
-      </c>
+        <v>9.624688900321285</v>
+      </c>
+      <c r="O52" s="16"/>
+      <c r="P52" s="16"/>
+      <c r="Q52" s="16"/>
+      <c r="R52" s="16"/>
     </row>
-    <row r="53" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C53" s="20">
         <v>45720</v>
       </c>
@@ -39269,19 +39461,23 @@
         <v>2.3809999999999998</v>
       </c>
       <c r="K53" s="16">
-        <v>10.126453418843138</v>
+        <v>11.45105752280781</v>
       </c>
       <c r="L53" s="16">
-        <v>3.3723793103448272</v>
+        <v>3.6240987034648779</v>
       </c>
       <c r="M53" s="16">
-        <v>40.420375681210324</v>
+        <v>62.085780463657926</v>
       </c>
       <c r="N53" s="16">
-        <v>7.2498498903165149</v>
-      </c>
+        <v>9.9535581101728514</v>
+      </c>
+      <c r="O53" s="16"/>
+      <c r="P53" s="16"/>
+      <c r="Q53" s="16"/>
+      <c r="R53" s="16"/>
     </row>
-    <row r="54" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C54" s="20">
         <v>45809</v>
       </c>
@@ -39304,19 +39500,23 @@
         <v>2.4700000000000002</v>
       </c>
       <c r="K54" s="16">
-        <v>11.772334234729522</v>
+        <v>11.602478381355564</v>
       </c>
       <c r="L54" s="16">
-        <v>3.6384662032243753</v>
+        <v>3.6571179389122035</v>
       </c>
       <c r="M54" s="16">
-        <v>84.339689195489072</v>
+        <v>63.017071231097958</v>
       </c>
       <c r="N54" s="16">
-        <v>12.753651659845385</v>
-      </c>
+        <v>10.067691635637576</v>
+      </c>
+      <c r="O54" s="16"/>
+      <c r="P54" s="16"/>
+      <c r="Q54" s="16"/>
+      <c r="R54" s="16"/>
     </row>
-    <row r="55" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:18" x14ac:dyDescent="0.3">
       <c r="C55" s="20">
         <v>45871</v>
       </c>
@@ -39350,6 +39550,10 @@
       <c r="N55" s="16">
         <v>9.1723716275683067</v>
       </c>
+      <c r="O55" s="16"/>
+      <c r="P55" s="16"/>
+      <c r="Q55" s="16"/>
+      <c r="R55" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>